<commit_message>
Add final judgements and suggestions at the end of the report
</commit_message>
<xml_diff>
--- a/report_template_simplified.xlsx
+++ b/report_template_simplified.xlsx
@@ -96,11 +96,12 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -119,6 +120,13 @@
     </font>
     <font>
       <sz val="13"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -200,31 +208,31 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -262,7 +270,7 @@
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FFFFD8CE"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -272,13 +280,13 @@
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FF80FF80"/>
       <rgbColor rgb="FFDDE8CB"/>
       <rgbColor rgb="FFFFFF99"/>
-      <rgbColor rgb="FF80FF80"/>
+      <rgbColor rgb="FFA0E0A0"/>
       <rgbColor rgb="FFEC9BA4"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFD8CE"/>
+      <rgbColor rgb="FFFFC080"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
@@ -287,13 +295,13 @@
       <rgbColor rgb="FFFF6600"/>
       <rgbColor rgb="FF666699"/>
       <rgbColor rgb="FFB3B3B3"/>
-      <rgbColor rgb="FF004586"/>
-      <rgbColor rgb="FF50938A"/>
+      <rgbColor rgb="FF004080"/>
+      <rgbColor rgb="FF40C040"/>
       <rgbColor rgb="FF003300"/>
       <rgbColor rgb="FF333300"/>
       <rgbColor rgb="FF993300"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FF355269"/>
+      <rgbColor rgb="FF004586"/>
       <rgbColor rgb="FF333333"/>
     </indexedColors>
   </colors>
@@ -319,8 +327,12 @@
             </a:pPr>
             <a:r>
               <a:rPr sz="1300" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:rPr>
               <a:t>Pilastri ESG</a:t>
             </a:r>
@@ -396,7 +408,7 @@
             <c:invertIfNegative val="0"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="50938A"/>
+                <a:srgbClr val="40C040"/>
               </a:solidFill>
               <a:ln w="0">
                 <a:solidFill>
@@ -410,7 +422,7 @@
             <c:invertIfNegative val="0"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="EC9BA4"/>
+                <a:srgbClr val="FFC080"/>
               </a:solidFill>
               <a:ln w="0">
                 <a:solidFill>
@@ -424,7 +436,7 @@
             <c:invertIfNegative val="0"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="355269"/>
+                <a:srgbClr val="004080"/>
               </a:solidFill>
               <a:ln w="0">
                 <a:solidFill>
@@ -442,8 +454,12 @@
                 <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
                       <a:uFillTx/>
                       <a:latin typeface="Arial"/>
+                      <a:ea typeface="DejaVu Sans"/>
                     </a:defRPr>
                   </a:pPr>
                 </a:p>
@@ -463,8 +479,12 @@
                 <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
                       <a:uFillTx/>
                       <a:latin typeface="Arial"/>
+                      <a:ea typeface="DejaVu Sans"/>
                     </a:defRPr>
                   </a:pPr>
                 </a:p>
@@ -484,8 +504,12 @@
                 <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
                       <a:uFillTx/>
                       <a:latin typeface="Arial"/>
+                      <a:ea typeface="DejaVu Sans"/>
                     </a:defRPr>
                   </a:pPr>
                 </a:p>
@@ -503,8 +527,12 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
+                    <a:ea typeface="DejaVu Sans"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
@@ -569,18 +597,18 @@
         </c:ser>
         <c:gapWidth val="100"/>
         <c:shape val="box"/>
-        <c:axId val="26756993"/>
-        <c:axId val="30589095"/>
+        <c:axId val="57980357"/>
+        <c:axId val="27227936"/>
         <c:axId val="0"/>
       </c:bar3DChart>
       <c:catAx>
-        <c:axId val="26756993"/>
+        <c:axId val="57980357"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -597,13 +625,17 @@
           <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="30589095"/>
+        <c:crossAx val="27227936"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -611,7 +643,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="30589095"/>
+        <c:axId val="27227936"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="100"/>
@@ -627,7 +659,7 @@
             </a:ln>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -644,13 +676,17 @@
           <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="26756993"/>
+        <c:crossAx val="57980357"/>
         <c:crossesAt val="1"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -688,8 +724,12 @@
             </a:pPr>
             <a:r>
               <a:rPr sz="1300" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:rPr>
               <a:t>Grado di priorità per ESRS specifico</a:t>
             </a:r>
@@ -765,7 +805,7 @@
             <c:invertIfNegative val="0"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="50938A"/>
+                <a:srgbClr val="40C040"/>
               </a:solidFill>
               <a:ln w="0">
                 <a:solidFill>
@@ -779,7 +819,7 @@
             <c:invertIfNegative val="0"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="50938A"/>
+                <a:srgbClr val="40C040"/>
               </a:solidFill>
               <a:ln w="0">
                 <a:solidFill>
@@ -793,7 +833,7 @@
             <c:invertIfNegative val="0"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="50938A"/>
+                <a:srgbClr val="40C040"/>
               </a:solidFill>
               <a:ln w="0">
                 <a:solidFill>
@@ -807,7 +847,7 @@
             <c:invertIfNegative val="0"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="50938A"/>
+                <a:srgbClr val="40C040"/>
               </a:solidFill>
               <a:ln w="0">
                 <a:solidFill>
@@ -821,7 +861,7 @@
             <c:invertIfNegative val="0"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="50938A"/>
+                <a:srgbClr val="40C040"/>
               </a:solidFill>
               <a:ln w="0">
                 <a:solidFill>
@@ -835,7 +875,7 @@
             <c:invertIfNegative val="0"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="EC9BA4"/>
+                <a:srgbClr val="FFC080"/>
               </a:solidFill>
               <a:ln w="0">
                 <a:solidFill>
@@ -849,7 +889,7 @@
             <c:invertIfNegative val="0"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="EC9BA4"/>
+                <a:srgbClr val="FFC080"/>
               </a:solidFill>
               <a:ln w="0">
                 <a:solidFill>
@@ -863,7 +903,7 @@
             <c:invertIfNegative val="0"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="EC9BA4"/>
+                <a:srgbClr val="FFC080"/>
               </a:solidFill>
               <a:ln w="0">
                 <a:solidFill>
@@ -877,7 +917,7 @@
             <c:invertIfNegative val="0"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="EC9BA4"/>
+                <a:srgbClr val="FFC080"/>
               </a:solidFill>
               <a:ln w="0">
                 <a:solidFill>
@@ -891,7 +931,7 @@
             <c:invertIfNegative val="0"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="355269"/>
+                <a:srgbClr val="004080"/>
               </a:solidFill>
               <a:ln w="0">
                 <a:solidFill>
@@ -909,8 +949,12 @@
                 <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
                       <a:uFillTx/>
                       <a:latin typeface="Arial"/>
+                      <a:ea typeface="DejaVu Sans"/>
                     </a:defRPr>
                   </a:pPr>
                 </a:p>
@@ -930,8 +974,12 @@
                 <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
                       <a:uFillTx/>
                       <a:latin typeface="Arial"/>
+                      <a:ea typeface="DejaVu Sans"/>
                     </a:defRPr>
                   </a:pPr>
                 </a:p>
@@ -951,8 +999,12 @@
                 <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
                       <a:uFillTx/>
                       <a:latin typeface="Arial"/>
+                      <a:ea typeface="DejaVu Sans"/>
                     </a:defRPr>
                   </a:pPr>
                 </a:p>
@@ -972,8 +1024,12 @@
                 <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
                       <a:uFillTx/>
                       <a:latin typeface="Arial"/>
+                      <a:ea typeface="DejaVu Sans"/>
                     </a:defRPr>
                   </a:pPr>
                 </a:p>
@@ -993,8 +1049,12 @@
                 <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
                       <a:uFillTx/>
                       <a:latin typeface="Arial"/>
+                      <a:ea typeface="DejaVu Sans"/>
                     </a:defRPr>
                   </a:pPr>
                 </a:p>
@@ -1014,8 +1074,12 @@
                 <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
                       <a:uFillTx/>
                       <a:latin typeface="Arial"/>
+                      <a:ea typeface="DejaVu Sans"/>
                     </a:defRPr>
                   </a:pPr>
                 </a:p>
@@ -1035,8 +1099,12 @@
                 <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
                       <a:uFillTx/>
                       <a:latin typeface="Arial"/>
+                      <a:ea typeface="DejaVu Sans"/>
                     </a:defRPr>
                   </a:pPr>
                 </a:p>
@@ -1056,8 +1124,12 @@
                 <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
                       <a:uFillTx/>
                       <a:latin typeface="Arial"/>
+                      <a:ea typeface="DejaVu Sans"/>
                     </a:defRPr>
                   </a:pPr>
                 </a:p>
@@ -1077,8 +1149,12 @@
                 <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
                       <a:uFillTx/>
                       <a:latin typeface="Arial"/>
+                      <a:ea typeface="DejaVu Sans"/>
                     </a:defRPr>
                   </a:pPr>
                 </a:p>
@@ -1098,8 +1174,12 @@
                 <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
                       <a:uFillTx/>
                       <a:latin typeface="Arial"/>
+                      <a:ea typeface="DejaVu Sans"/>
                     </a:defRPr>
                   </a:pPr>
                 </a:p>
@@ -1117,8 +1197,12 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
+                    <a:ea typeface="DejaVu Sans"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
@@ -1225,18 +1309,18 @@
         </c:ser>
         <c:gapWidth val="100"/>
         <c:shape val="box"/>
-        <c:axId val="75739719"/>
-        <c:axId val="29186266"/>
+        <c:axId val="39084625"/>
+        <c:axId val="58546082"/>
         <c:axId val="0"/>
       </c:bar3DChart>
       <c:catAx>
-        <c:axId val="75739719"/>
+        <c:axId val="39084625"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1253,13 +1337,17 @@
           <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="29186266"/>
+        <c:crossAx val="58546082"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1267,7 +1355,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="29186266"/>
+        <c:axId val="58546082"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="100"/>
@@ -1283,7 +1371,7 @@
             </a:ln>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1300,13 +1388,17 @@
           <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="75739719"/>
+        <c:crossAx val="39084625"/>
         <c:crossesAt val="1"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1344,8 +1436,12 @@
             </a:pPr>
             <a:r>
               <a:rPr sz="1300" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:rPr>
               <a:t>Prioritizzazione delle categorie</a:t>
             </a:r>
@@ -1370,11 +1466,11 @@
           <c:order val="0"/>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="50938A"/>
+              <a:srgbClr val="008000"/>
             </a:solidFill>
             <a:ln w="28800">
               <a:solidFill>
-                <a:srgbClr val="50938A"/>
+                <a:srgbClr val="008000"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -1384,7 +1480,7 @@
             <c:size val="8"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="50938A"/>
+                <a:srgbClr val="008000"/>
               </a:solidFill>
             </c:spPr>
           </c:marker>
@@ -1395,8 +1491,12 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
+                    <a:ea typeface="DejaVu Sans"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
@@ -1471,17 +1571,66 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="33938408"/>
-        <c:axId val="5945699"/>
+        <c:axId val="63606581"/>
+        <c:axId val="60085722"/>
       </c:radarChart>
       <c:catAx>
-        <c:axId val="33938408"/>
+        <c:axId val="63606581"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="0">
+            <a:noFill/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:uFillTx/>
+                <a:latin typeface="Arial"/>
+                <a:ea typeface="DejaVu Sans"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="60085722"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="60085722"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="100"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="0">
+              <a:solidFill>
+                <a:srgbClr val="B3B3B3"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1498,60 +1647,17 @@
           <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="5945699"/>
-        <c:crosses val="autoZero"/>
-        <c:auto val="1"/>
-        <c:lblAlgn val="ctr"/>
-        <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
-      </c:catAx>
-      <c:valAx>
-        <c:axId val="5945699"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-          <c:max val="100"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="0">
-              <a:solidFill>
-                <a:srgbClr val="B3B3B3"/>
-              </a:solidFill>
-            </a:ln>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="out"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:ln w="0">
-            <a:solidFill>
-              <a:srgbClr val="B3B3B3"/>
-            </a:solidFill>
-          </a:ln>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
-                <a:uFillTx/>
-                <a:latin typeface="Arial"/>
-              </a:defRPr>
-            </a:pPr>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="33938408"/>
+        <c:crossAx val="63606581"/>
         <c:crossesAt val="1"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1595,8 +1701,12 @@
             </a:pPr>
             <a:r>
               <a:rPr sz="1300" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:rPr>
               <a:t>Distribuzione delle risposte al questionario</a:t>
             </a:r>
@@ -1669,12 +1779,17 @@
                 <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
                       <a:uFillTx/>
                       <a:latin typeface="Arial"/>
+                      <a:ea typeface="DejaVu Sans"/>
                     </a:defRPr>
                   </a:pPr>
                 </a:p>
               </c:txPr>
+              <c:dLblPos val="bestFit"/>
               <c:showLegendKey val="0"/>
               <c:showVal val="0"/>
               <c:showCatName val="0"/>
@@ -1690,12 +1805,17 @@
                 <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
                       <a:uFillTx/>
                       <a:latin typeface="Arial"/>
+                      <a:ea typeface="DejaVu Sans"/>
                     </a:defRPr>
                   </a:pPr>
                 </a:p>
               </c:txPr>
+              <c:dLblPos val="bestFit"/>
               <c:showLegendKey val="0"/>
               <c:showVal val="0"/>
               <c:showCatName val="0"/>
@@ -1711,12 +1831,17 @@
                 <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
                       <a:uFillTx/>
                       <a:latin typeface="Arial"/>
+                      <a:ea typeface="DejaVu Sans"/>
                     </a:defRPr>
                   </a:pPr>
                 </a:p>
               </c:txPr>
+              <c:dLblPos val="bestFit"/>
               <c:showLegendKey val="0"/>
               <c:showVal val="0"/>
               <c:showCatName val="0"/>
@@ -1730,12 +1855,17 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
+                    <a:ea typeface="DejaVu Sans"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="bestFit"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
@@ -1813,14 +1943,341 @@
         <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
               <a:uFillTx/>
               <a:latin typeface="Arial"/>
+              <a:ea typeface="DejaVu Sans"/>
             </a:defRPr>
           </a:pPr>
         </a:p>
       </c:txPr>
     </c:legend>
     <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="zero"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln w="0">
+      <a:noFill/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1300" b="0" u="none" strike="noStrike">
+                <a:uFillTx/>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr sz="1300" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:uFillTx/>
+                <a:latin typeface="Arial"/>
+                <a:ea typeface="DejaVu Sans"/>
+              </a:rPr>
+              <a:t>Punteggio complessivo</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:view3D>
+      <c:rotX val="11"/>
+      <c:rotY val="25"/>
+      <c:rAngAx val="1"/>
+      <c:perspective val="40"/>
+    </c:view3D>
+    <c:floor>
+      <c:spPr>
+        <a:solidFill>
+          <a:srgbClr val="CCCCCC"/>
+        </a:solidFill>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:floor>
+    <c:sideWall>
+      <c:spPr>
+        <a:solidFill>
+          <a:srgbClr val="A0E0A0"/>
+        </a:solidFill>
+        <a:ln w="0">
+          <a:solidFill>
+            <a:srgbClr val="B3B3B3"/>
+          </a:solidFill>
+        </a:ln>
+      </c:spPr>
+    </c:sideWall>
+    <c:backWall>
+      <c:spPr>
+        <a:solidFill>
+          <a:srgbClr val="A0E0A0"/>
+        </a:solidFill>
+        <a:ln w="0">
+          <a:solidFill>
+            <a:srgbClr val="B3B3B3"/>
+          </a:solidFill>
+        </a:ln>
+      </c:spPr>
+    </c:backWall>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.1875"/>
+          <c:y val="0.191666666666667"/>
+          <c:w val="0.62490625"/>
+          <c:h val="0.666166666666667"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:bar3DChart>
+        <c:barDir val="bar"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Foglio1!$A$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Punteggio complessivo</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="004586"/>
+            </a:solidFill>
+            <a:ln w="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:invertIfNegative val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="EEEEEE"/>
+              </a:solidFill>
+              <a:ln w="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dLbls>
+            <c:dLbl>
+              <c:idx val="0"/>
+              <c:txPr>
+                <a:bodyPr wrap="none"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
+                      <a:uFillTx/>
+                      <a:latin typeface="Arial"/>
+                      <a:ea typeface="DejaVu Sans"/>
+                    </a:defRPr>
+                  </a:pPr>
+                </a:p>
+              </c:txPr>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:separator> </c:separator>
+            </c:dLbl>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:uFillTx/>
+                    <a:latin typeface="Arial"/>
+                    <a:ea typeface="DejaVu Sans"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:leaderLines>
+              <c:spPr>
+                <a:ln w="0">
+                  <a:solidFill>
+                    <a:srgbClr val="000000"/>
+                  </a:solidFill>
+                </a:ln>
+              </c:spPr>
+            </c:leaderLines>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:val>
+            <c:numRef>
+              <c:f>Foglio1!$B$1</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>50</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="100"/>
+        <c:shape val="box"/>
+        <c:axId val="61365308"/>
+        <c:axId val="66388280"/>
+        <c:axId val="0"/>
+      </c:bar3DChart>
+      <c:catAx>
+        <c:axId val="61365308"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="0">
+            <a:solidFill>
+              <a:srgbClr val="B3B3B3"/>
+            </a:solidFill>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:uFillTx/>
+                <a:latin typeface="Arial"/>
+                <a:ea typeface="DejaVu Sans"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="66388280"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="66388280"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="100"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="0">
+              <a:solidFill>
+                <a:srgbClr val="B3B3B3"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="0">
+            <a:solidFill>
+              <a:srgbClr val="B3B3B3"/>
+            </a:solidFill>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:uFillTx/>
+                <a:latin typeface="Arial"/>
+                <a:ea typeface="DejaVu Sans"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="61365308"/>
+        <c:crossesAt val="0"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1857,13 +2314,21 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="419">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor"/>
+    <cs:lineWidthScale>1</cs:lineWidthScale>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+    <a:defRPr sz="1800" b="0"/>
   </cs:axisTitle>
   <cs:categoryAxis>
     <cs:lnRef idx="0"/>
@@ -2071,9 +2536,11 @@
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="419">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor"/>
+    <cs:lineWidthScale>1</cs:lineWidthScale>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+    <a:defRPr sz="1800" b="0"/>
   </cs:axisTitle>
   <cs:categoryAxis>
     <cs:lnRef idx="0"/>
@@ -2281,9 +2748,11 @@
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="419">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor"/>
+    <cs:lineWidthScale>1</cs:lineWidthScale>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+    <a:defRPr sz="1800" b="0"/>
   </cs:axisTitle>
   <cs:categoryAxis>
     <cs:lnRef idx="0"/>
@@ -2491,9 +2960,11 @@
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="419">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor"/>
+    <cs:lineWidthScale>1</cs:lineWidthScale>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+    <a:defRPr sz="1800" b="0"/>
   </cs:axisTitle>
   <cs:categoryAxis>
     <cs:lnRef idx="0"/>
@@ -2697,6 +3168,218 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="419">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:lineWidthScale>1</cs:lineWidthScale>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+    <a:defRPr sz="1800" b="0"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataLabel>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <cs:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataPointMarkerLayout>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:legend>
+  <cs:plotArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:plotArea>
+  <cs:plotArea3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
@@ -2708,9 +3391,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>78840</xdr:colOff>
+      <xdr:colOff>79560</xdr:colOff>
       <xdr:row>20</xdr:row>
-      <xdr:rowOff>1080</xdr:rowOff>
+      <xdr:rowOff>360</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2719,7 +3402,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="0" y="0"/>
-        <a:ext cx="5759640" cy="3239640"/>
+        <a:ext cx="5758920" cy="3238920"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2738,9 +3421,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>149400</xdr:colOff>
+      <xdr:colOff>148320</xdr:colOff>
       <xdr:row>20</xdr:row>
-      <xdr:rowOff>1080</xdr:rowOff>
+      <xdr:rowOff>360</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2748,8 +3431,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="5760000" y="0"/>
-        <a:ext cx="5759640" cy="3239640"/>
+        <a:off x="5758560" y="0"/>
+        <a:ext cx="5758920" cy="3238920"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2768,9 +3451,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>78840</xdr:colOff>
+      <xdr:colOff>79560</xdr:colOff>
       <xdr:row>40</xdr:row>
-      <xdr:rowOff>2520</xdr:rowOff>
+      <xdr:rowOff>1800</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2779,7 +3462,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="0" y="3240000"/>
-        <a:ext cx="5759640" cy="3239640"/>
+        <a:ext cx="5758920" cy="3238920"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2798,9 +3481,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>149400</xdr:colOff>
+      <xdr:colOff>148320</xdr:colOff>
       <xdr:row>40</xdr:row>
-      <xdr:rowOff>2520</xdr:rowOff>
+      <xdr:rowOff>1800</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2808,12 +3491,42 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="5760000" y="3240000"/>
-        <a:ext cx="5759640" cy="3239640"/>
+        <a:off x="5758560" y="3240000"/>
+        <a:ext cx="5758920" cy="3238920"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>2880</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>150480</xdr:colOff>
+      <xdr:row>53</xdr:row>
+      <xdr:rowOff>57600</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name=""/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="6480000"/>
+        <a:ext cx="11519640" cy="2159640"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2933,44 +3646,31 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AB115"/>
+  <dimension ref="A1:M115"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.39"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="11.53"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="6" min="4" style="1" width="11.53"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="28" min="7" style="2" width="11.53"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="49" min="29" style="1" width="11.53"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="50" style="2" width="11.53"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="4" style="1" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="n">
+      <c r="B1" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="D1" s="0"/>
-      <c r="E1" s="0"/>
-      <c r="F1" s="0"/>
-      <c r="G1" s="0"/>
-      <c r="H1" s="0"/>
-      <c r="I1" s="0"/>
-      <c r="J1" s="0"/>
-      <c r="K1" s="0"/>
-      <c r="L1" s="0"/>
-      <c r="M1" s="0"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
-      <c r="P1" s="1"/>
-      <c r="Q1" s="1"/>
-      <c r="R1" s="1"/>
-      <c r="X1" s="1"/>
-      <c r="Y1" s="1"/>
-      <c r="Z1" s="1"/>
-      <c r="AA1" s="1"/>
-      <c r="AB1" s="1"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="L1" s="3"/>
+      <c r="M1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
@@ -2979,26 +3679,16 @@
       <c r="B2" s="4" t="n">
         <v>33</v>
       </c>
-      <c r="D2" s="0"/>
-      <c r="E2" s="0"/>
-      <c r="F2" s="0"/>
-      <c r="G2" s="0"/>
-      <c r="H2" s="0"/>
-      <c r="I2" s="0"/>
-      <c r="J2" s="0"/>
-      <c r="K2" s="0"/>
-      <c r="L2" s="0"/>
-      <c r="M2" s="0"/>
-      <c r="N2" s="1"/>
-      <c r="O2" s="1"/>
-      <c r="P2" s="1"/>
-      <c r="Q2" s="1"/>
-      <c r="R2" s="1"/>
-      <c r="X2" s="1"/>
-      <c r="Y2" s="1"/>
-      <c r="Z2" s="1"/>
-      <c r="AA2" s="1"/>
-      <c r="AB2" s="1"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
@@ -3007,26 +3697,16 @@
       <c r="B3" s="4" t="n">
         <v>33</v>
       </c>
-      <c r="D3" s="0"/>
-      <c r="E3" s="0"/>
-      <c r="F3" s="0"/>
-      <c r="G3" s="0"/>
-      <c r="H3" s="0"/>
-      <c r="I3" s="0"/>
-      <c r="J3" s="0"/>
-      <c r="K3" s="0"/>
-      <c r="L3" s="0"/>
-      <c r="M3" s="0"/>
-      <c r="N3" s="1"/>
-      <c r="O3" s="1"/>
-      <c r="P3" s="1"/>
-      <c r="Q3" s="1"/>
-      <c r="R3" s="1"/>
-      <c r="X3" s="1"/>
-      <c r="Y3" s="1"/>
-      <c r="Z3" s="1"/>
-      <c r="AA3" s="1"/>
-      <c r="AB3" s="1"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="M3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
@@ -3035,26 +3715,16 @@
       <c r="B4" s="4" t="n">
         <v>33</v>
       </c>
-      <c r="D4" s="0"/>
-      <c r="E4" s="0"/>
-      <c r="F4" s="0"/>
-      <c r="G4" s="0"/>
-      <c r="H4" s="0"/>
-      <c r="I4" s="0"/>
-      <c r="J4" s="0"/>
-      <c r="K4" s="0"/>
-      <c r="L4" s="0"/>
-      <c r="M4" s="0"/>
-      <c r="N4" s="1"/>
-      <c r="O4" s="1"/>
-      <c r="P4" s="1"/>
-      <c r="Q4" s="1"/>
-      <c r="R4" s="1"/>
-      <c r="X4" s="1"/>
-      <c r="Y4" s="1"/>
-      <c r="Z4" s="1"/>
-      <c r="AA4" s="1"/>
-      <c r="AB4" s="1"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+      <c r="M4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
@@ -3063,26 +3733,16 @@
       <c r="B5" s="5" t="n">
         <v>25</v>
       </c>
-      <c r="D5" s="0"/>
-      <c r="E5" s="0"/>
-      <c r="F5" s="0"/>
-      <c r="G5" s="0"/>
-      <c r="H5" s="0"/>
-      <c r="I5" s="0"/>
-      <c r="J5" s="0"/>
-      <c r="K5" s="0"/>
-      <c r="L5" s="0"/>
-      <c r="M5" s="0"/>
-      <c r="N5" s="1"/>
-      <c r="O5" s="1"/>
-      <c r="P5" s="1"/>
-      <c r="Q5" s="1"/>
-      <c r="R5" s="1"/>
-      <c r="X5" s="1"/>
-      <c r="Y5" s="1"/>
-      <c r="Z5" s="1"/>
-      <c r="AA5" s="1"/>
-      <c r="AB5" s="1"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+      <c r="L5" s="3"/>
+      <c r="M5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
@@ -3091,26 +3751,16 @@
       <c r="B6" s="5" t="n">
         <v>25</v>
       </c>
-      <c r="D6" s="0"/>
-      <c r="E6" s="0"/>
-      <c r="F6" s="0"/>
-      <c r="G6" s="0"/>
-      <c r="H6" s="0"/>
-      <c r="I6" s="0"/>
-      <c r="J6" s="0"/>
-      <c r="K6" s="0"/>
-      <c r="L6" s="0"/>
-      <c r="M6" s="0"/>
-      <c r="N6" s="1"/>
-      <c r="O6" s="1"/>
-      <c r="P6" s="1"/>
-      <c r="Q6" s="1"/>
-      <c r="R6" s="1"/>
-      <c r="X6" s="1"/>
-      <c r="Y6" s="1"/>
-      <c r="Z6" s="1"/>
-      <c r="AA6" s="1"/>
-      <c r="AB6" s="1"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
+      <c r="K6" s="3"/>
+      <c r="L6" s="3"/>
+      <c r="M6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
@@ -3119,26 +3769,16 @@
       <c r="B7" s="5" t="n">
         <v>25</v>
       </c>
-      <c r="D7" s="0"/>
-      <c r="E7" s="0"/>
-      <c r="F7" s="0"/>
-      <c r="G7" s="0"/>
-      <c r="H7" s="0"/>
-      <c r="I7" s="0"/>
-      <c r="J7" s="0"/>
-      <c r="K7" s="0"/>
-      <c r="L7" s="0"/>
-      <c r="M7" s="0"/>
-      <c r="N7" s="1"/>
-      <c r="O7" s="1"/>
-      <c r="P7" s="1"/>
-      <c r="Q7" s="1"/>
-      <c r="R7" s="1"/>
-      <c r="X7" s="1"/>
-      <c r="Y7" s="1"/>
-      <c r="Z7" s="1"/>
-      <c r="AA7" s="1"/>
-      <c r="AB7" s="1"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3"/>
+      <c r="L7" s="3"/>
+      <c r="M7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
@@ -3147,26 +3787,16 @@
       <c r="B8" s="5" t="n">
         <v>25</v>
       </c>
-      <c r="D8" s="0"/>
-      <c r="E8" s="0"/>
-      <c r="F8" s="0"/>
-      <c r="G8" s="0"/>
-      <c r="H8" s="0"/>
-      <c r="I8" s="0"/>
-      <c r="J8" s="0"/>
-      <c r="K8" s="0"/>
-      <c r="L8" s="0"/>
-      <c r="M8" s="0"/>
-      <c r="N8" s="1"/>
-      <c r="O8" s="1"/>
-      <c r="P8" s="1"/>
-      <c r="Q8" s="1"/>
-      <c r="R8" s="1"/>
-      <c r="X8" s="1"/>
-      <c r="Y8" s="1"/>
-      <c r="Z8" s="1"/>
-      <c r="AA8" s="1"/>
-      <c r="AB8" s="1"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+      <c r="L8" s="3"/>
+      <c r="M8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
@@ -3175,26 +3805,16 @@
       <c r="B9" s="5" t="n">
         <v>25</v>
       </c>
-      <c r="D9" s="0"/>
-      <c r="E9" s="0"/>
-      <c r="F9" s="0"/>
-      <c r="G9" s="0"/>
-      <c r="H9" s="0"/>
-      <c r="I9" s="0"/>
-      <c r="J9" s="0"/>
-      <c r="K9" s="0"/>
-      <c r="L9" s="0"/>
-      <c r="M9" s="0"/>
-      <c r="N9" s="1"/>
-      <c r="O9" s="1"/>
-      <c r="P9" s="1"/>
-      <c r="Q9" s="1"/>
-      <c r="R9" s="1"/>
-      <c r="X9" s="1"/>
-      <c r="Y9" s="1"/>
-      <c r="Z9" s="1"/>
-      <c r="AA9" s="1"/>
-      <c r="AB9" s="1"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="3"/>
+      <c r="K9" s="3"/>
+      <c r="L9" s="3"/>
+      <c r="M9" s="3"/>
     </row>
     <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
@@ -3203,26 +3823,16 @@
       <c r="B10" s="5" t="n">
         <v>25</v>
       </c>
-      <c r="D10" s="0"/>
-      <c r="E10" s="0"/>
-      <c r="F10" s="0"/>
-      <c r="G10" s="0"/>
-      <c r="H10" s="0"/>
-      <c r="I10" s="0"/>
-      <c r="J10" s="0"/>
-      <c r="K10" s="0"/>
-      <c r="L10" s="0"/>
-      <c r="M10" s="0"/>
-      <c r="N10" s="1"/>
-      <c r="O10" s="1"/>
-      <c r="P10" s="1"/>
-      <c r="Q10" s="1"/>
-      <c r="R10" s="1"/>
-      <c r="X10" s="1"/>
-      <c r="Y10" s="1"/>
-      <c r="Z10" s="1"/>
-      <c r="AA10" s="1"/>
-      <c r="AB10" s="1"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3"/>
+      <c r="K10" s="3"/>
+      <c r="L10" s="3"/>
+      <c r="M10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
@@ -3231,26 +3841,16 @@
       <c r="B11" s="5" t="n">
         <v>25</v>
       </c>
-      <c r="D11" s="0"/>
-      <c r="E11" s="0"/>
-      <c r="F11" s="0"/>
-      <c r="G11" s="0"/>
-      <c r="H11" s="0"/>
-      <c r="I11" s="0"/>
-      <c r="J11" s="0"/>
-      <c r="K11" s="0"/>
-      <c r="L11" s="0"/>
-      <c r="M11" s="0"/>
-      <c r="N11" s="1"/>
-      <c r="O11" s="1"/>
-      <c r="P11" s="1"/>
-      <c r="Q11" s="1"/>
-      <c r="R11" s="1"/>
-      <c r="X11" s="1"/>
-      <c r="Y11" s="1"/>
-      <c r="Z11" s="1"/>
-      <c r="AA11" s="1"/>
-      <c r="AB11" s="1"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3"/>
+      <c r="J11" s="3"/>
+      <c r="K11" s="3"/>
+      <c r="L11" s="3"/>
+      <c r="M11" s="3"/>
     </row>
     <row r="12" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
@@ -3259,26 +3859,16 @@
       <c r="B12" s="5" t="n">
         <v>25</v>
       </c>
-      <c r="D12" s="0"/>
-      <c r="E12" s="0"/>
-      <c r="F12" s="0"/>
-      <c r="G12" s="0"/>
-      <c r="H12" s="0"/>
-      <c r="I12" s="0"/>
-      <c r="J12" s="0"/>
-      <c r="K12" s="0"/>
-      <c r="L12" s="0"/>
-      <c r="M12" s="0"/>
-      <c r="N12" s="1"/>
-      <c r="O12" s="1"/>
-      <c r="P12" s="1"/>
-      <c r="Q12" s="1"/>
-      <c r="R12" s="1"/>
-      <c r="X12" s="1"/>
-      <c r="Y12" s="1"/>
-      <c r="Z12" s="1"/>
-      <c r="AA12" s="1"/>
-      <c r="AB12" s="1"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3"/>
+      <c r="J12" s="3"/>
+      <c r="K12" s="3"/>
+      <c r="L12" s="3"/>
+      <c r="M12" s="3"/>
     </row>
     <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
@@ -3287,26 +3877,16 @@
       <c r="B13" s="5" t="n">
         <v>25</v>
       </c>
-      <c r="D13" s="0"/>
-      <c r="E13" s="0"/>
-      <c r="F13" s="0"/>
-      <c r="G13" s="0"/>
-      <c r="H13" s="0"/>
-      <c r="I13" s="0"/>
-      <c r="J13" s="0"/>
-      <c r="K13" s="0"/>
-      <c r="L13" s="0"/>
-      <c r="M13" s="0"/>
-      <c r="N13" s="1"/>
-      <c r="O13" s="1"/>
-      <c r="P13" s="1"/>
-      <c r="Q13" s="1"/>
-      <c r="R13" s="1"/>
-      <c r="X13" s="1"/>
-      <c r="Y13" s="1"/>
-      <c r="Z13" s="1"/>
-      <c r="AA13" s="1"/>
-      <c r="AB13" s="1"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3"/>
+      <c r="J13" s="3"/>
+      <c r="K13" s="3"/>
+      <c r="L13" s="3"/>
+      <c r="M13" s="3"/>
     </row>
     <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
@@ -3315,26 +3895,16 @@
       <c r="B14" s="5" t="n">
         <v>25</v>
       </c>
-      <c r="D14" s="0"/>
-      <c r="E14" s="0"/>
-      <c r="F14" s="0"/>
-      <c r="G14" s="0"/>
-      <c r="H14" s="0"/>
-      <c r="I14" s="0"/>
-      <c r="J14" s="0"/>
-      <c r="K14" s="0"/>
-      <c r="L14" s="0"/>
-      <c r="M14" s="0"/>
-      <c r="N14" s="1"/>
-      <c r="O14" s="1"/>
-      <c r="P14" s="1"/>
-      <c r="Q14" s="1"/>
-      <c r="R14" s="1"/>
-      <c r="X14" s="1"/>
-      <c r="Y14" s="1"/>
-      <c r="Z14" s="1"/>
-      <c r="AA14" s="1"/>
-      <c r="AB14" s="1"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+      <c r="J14" s="3"/>
+      <c r="K14" s="3"/>
+      <c r="L14" s="3"/>
+      <c r="M14" s="3"/>
     </row>
     <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
@@ -3343,26 +3913,16 @@
       <c r="B15" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="D15" s="0"/>
-      <c r="E15" s="0"/>
-      <c r="F15" s="0"/>
-      <c r="G15" s="0"/>
-      <c r="H15" s="0"/>
-      <c r="I15" s="0"/>
-      <c r="J15" s="0"/>
-      <c r="K15" s="0"/>
-      <c r="L15" s="0"/>
-      <c r="M15" s="0"/>
-      <c r="N15" s="1"/>
-      <c r="O15" s="1"/>
-      <c r="P15" s="1"/>
-      <c r="Q15" s="1"/>
-      <c r="R15" s="1"/>
-      <c r="X15" s="1"/>
-      <c r="Y15" s="1"/>
-      <c r="Z15" s="1"/>
-      <c r="AA15" s="1"/>
-      <c r="AB15" s="1"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3"/>
+      <c r="J15" s="3"/>
+      <c r="K15" s="3"/>
+      <c r="L15" s="3"/>
+      <c r="M15" s="3"/>
     </row>
     <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
@@ -3371,26 +3931,16 @@
       <c r="B16" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="D16" s="0"/>
-      <c r="E16" s="0"/>
-      <c r="F16" s="0"/>
-      <c r="G16" s="0"/>
-      <c r="H16" s="0"/>
-      <c r="I16" s="0"/>
-      <c r="J16" s="0"/>
-      <c r="K16" s="0"/>
-      <c r="L16" s="0"/>
-      <c r="M16" s="0"/>
-      <c r="N16" s="1"/>
-      <c r="O16" s="1"/>
-      <c r="P16" s="1"/>
-      <c r="Q16" s="1"/>
-      <c r="R16" s="1"/>
-      <c r="X16" s="1"/>
-      <c r="Y16" s="1"/>
-      <c r="Z16" s="1"/>
-      <c r="AA16" s="1"/>
-      <c r="AB16" s="1"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3"/>
+      <c r="I16" s="3"/>
+      <c r="J16" s="3"/>
+      <c r="K16" s="3"/>
+      <c r="L16" s="3"/>
+      <c r="M16" s="3"/>
     </row>
     <row r="17" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
@@ -3399,26 +3949,16 @@
       <c r="B17" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="D17" s="0"/>
-      <c r="E17" s="0"/>
-      <c r="F17" s="0"/>
-      <c r="G17" s="0"/>
-      <c r="H17" s="0"/>
-      <c r="I17" s="0"/>
-      <c r="J17" s="0"/>
-      <c r="K17" s="0"/>
-      <c r="L17" s="0"/>
-      <c r="M17" s="0"/>
-      <c r="N17" s="1"/>
-      <c r="O17" s="1"/>
-      <c r="P17" s="1"/>
-      <c r="Q17" s="1"/>
-      <c r="R17" s="1"/>
-      <c r="X17" s="1"/>
-      <c r="Y17" s="1"/>
-      <c r="Z17" s="1"/>
-      <c r="AA17" s="1"/>
-      <c r="AB17" s="1"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="3"/>
+      <c r="I17" s="3"/>
+      <c r="J17" s="3"/>
+      <c r="K17" s="3"/>
+      <c r="L17" s="3"/>
+      <c r="M17" s="3"/>
     </row>
     <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
@@ -3427,26 +3967,16 @@
       <c r="B18" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="D18" s="0"/>
-      <c r="E18" s="0"/>
-      <c r="F18" s="0"/>
-      <c r="G18" s="0"/>
-      <c r="H18" s="0"/>
-      <c r="I18" s="0"/>
-      <c r="J18" s="0"/>
-      <c r="K18" s="0"/>
-      <c r="L18" s="0"/>
-      <c r="M18" s="0"/>
-      <c r="N18" s="1"/>
-      <c r="O18" s="1"/>
-      <c r="P18" s="1"/>
-      <c r="Q18" s="1"/>
-      <c r="R18" s="1"/>
-      <c r="X18" s="1"/>
-      <c r="Y18" s="1"/>
-      <c r="Z18" s="1"/>
-      <c r="AA18" s="1"/>
-      <c r="AB18" s="1"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
+      <c r="I18" s="3"/>
+      <c r="J18" s="3"/>
+      <c r="K18" s="3"/>
+      <c r="L18" s="3"/>
+      <c r="M18" s="3"/>
     </row>
     <row r="19" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
@@ -3455,26 +3985,16 @@
       <c r="B19" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="D19" s="0"/>
-      <c r="E19" s="0"/>
-      <c r="F19" s="0"/>
-      <c r="G19" s="0"/>
-      <c r="H19" s="0"/>
-      <c r="I19" s="0"/>
-      <c r="J19" s="0"/>
-      <c r="K19" s="0"/>
-      <c r="L19" s="0"/>
-      <c r="M19" s="0"/>
-      <c r="N19" s="1"/>
-      <c r="O19" s="1"/>
-      <c r="P19" s="1"/>
-      <c r="Q19" s="1"/>
-      <c r="R19" s="1"/>
-      <c r="X19" s="1"/>
-      <c r="Y19" s="1"/>
-      <c r="Z19" s="1"/>
-      <c r="AA19" s="1"/>
-      <c r="AB19" s="1"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
+      <c r="I19" s="3"/>
+      <c r="J19" s="3"/>
+      <c r="K19" s="3"/>
+      <c r="L19" s="3"/>
+      <c r="M19" s="3"/>
     </row>
     <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
@@ -3483,26 +4003,16 @@
       <c r="B20" s="7" t="n">
         <v>25</v>
       </c>
-      <c r="D20" s="0"/>
-      <c r="E20" s="0"/>
-      <c r="F20" s="0"/>
-      <c r="G20" s="0"/>
-      <c r="H20" s="0"/>
-      <c r="I20" s="0"/>
-      <c r="J20" s="0"/>
-      <c r="K20" s="0"/>
-      <c r="L20" s="0"/>
-      <c r="M20" s="0"/>
-      <c r="N20" s="1"/>
-      <c r="O20" s="1"/>
-      <c r="P20" s="1"/>
-      <c r="Q20" s="1"/>
-      <c r="R20" s="1"/>
-      <c r="X20" s="1"/>
-      <c r="Y20" s="1"/>
-      <c r="Z20" s="1"/>
-      <c r="AA20" s="1"/>
-      <c r="AB20" s="1"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="3"/>
+      <c r="I20" s="3"/>
+      <c r="J20" s="3"/>
+      <c r="K20" s="3"/>
+      <c r="L20" s="3"/>
+      <c r="M20" s="3"/>
     </row>
     <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
@@ -3511,26 +4021,16 @@
       <c r="B21" s="7" t="n">
         <v>50</v>
       </c>
-      <c r="D21" s="0"/>
-      <c r="E21" s="0"/>
-      <c r="F21" s="0"/>
-      <c r="G21" s="0"/>
-      <c r="H21" s="0"/>
-      <c r="I21" s="0"/>
-      <c r="J21" s="0"/>
-      <c r="K21" s="0"/>
-      <c r="L21" s="0"/>
-      <c r="M21" s="0"/>
-      <c r="N21" s="1"/>
-      <c r="O21" s="1"/>
-      <c r="P21" s="1"/>
-      <c r="Q21" s="1"/>
-      <c r="R21" s="1"/>
-      <c r="X21" s="1"/>
-      <c r="Y21" s="1"/>
-      <c r="Z21" s="1"/>
-      <c r="AA21" s="1"/>
-      <c r="AB21" s="1"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
+      <c r="J21" s="3"/>
+      <c r="K21" s="3"/>
+      <c r="L21" s="3"/>
+      <c r="M21" s="3"/>
     </row>
     <row r="22" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
@@ -3539,1604 +4039,1077 @@
       <c r="B22" s="7" t="n">
         <v>25</v>
       </c>
-      <c r="D22" s="0"/>
-      <c r="E22" s="0"/>
-      <c r="F22" s="0"/>
-      <c r="G22" s="0"/>
-      <c r="H22" s="0"/>
-      <c r="I22" s="0"/>
-      <c r="J22" s="0"/>
-      <c r="K22" s="0"/>
-      <c r="L22" s="0"/>
-      <c r="M22" s="0"/>
-      <c r="N22" s="1"/>
-      <c r="O22" s="1"/>
-      <c r="P22" s="1"/>
-      <c r="Q22" s="1"/>
-      <c r="R22" s="1"/>
-      <c r="X22" s="1"/>
-      <c r="Y22" s="1"/>
-      <c r="Z22" s="1"/>
-      <c r="AA22" s="1"/>
-      <c r="AB22" s="1"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
+      <c r="I22" s="3"/>
+      <c r="J22" s="3"/>
+      <c r="K22" s="3"/>
+      <c r="L22" s="3"/>
+      <c r="M22" s="3"/>
     </row>
     <row r="23" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0"/>
-      <c r="B23" s="0"/>
-      <c r="D23" s="0"/>
-      <c r="E23" s="0"/>
-      <c r="F23" s="0"/>
-      <c r="G23" s="0"/>
-      <c r="H23" s="0"/>
-      <c r="I23" s="0"/>
-      <c r="J23" s="0"/>
-      <c r="K23" s="0"/>
-      <c r="L23" s="0"/>
-      <c r="M23" s="0"/>
-      <c r="N23" s="1"/>
-      <c r="O23" s="1"/>
-      <c r="P23" s="1"/>
-      <c r="Q23" s="1"/>
-      <c r="R23" s="1"/>
-      <c r="X23" s="1"/>
-      <c r="Y23" s="1"/>
-      <c r="Z23" s="1"/>
-      <c r="AA23" s="1"/>
-      <c r="AB23" s="1"/>
+      <c r="A23" s="3"/>
+      <c r="B23" s="3"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3"/>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
+      <c r="H23" s="3"/>
+      <c r="I23" s="3"/>
+      <c r="J23" s="3"/>
+      <c r="K23" s="3"/>
+      <c r="L23" s="3"/>
+      <c r="M23" s="3"/>
     </row>
     <row r="24" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0"/>
-      <c r="B24" s="0"/>
-      <c r="D24" s="0"/>
-      <c r="E24" s="0"/>
-      <c r="F24" s="0"/>
-      <c r="G24" s="0"/>
-      <c r="H24" s="0"/>
-      <c r="I24" s="0"/>
-      <c r="J24" s="0"/>
-      <c r="K24" s="0"/>
-      <c r="L24" s="0"/>
-      <c r="M24" s="0"/>
-      <c r="N24" s="1"/>
-      <c r="O24" s="1"/>
-      <c r="P24" s="1"/>
-      <c r="Q24" s="1"/>
-      <c r="R24" s="1"/>
-      <c r="X24" s="1"/>
-      <c r="Y24" s="1"/>
-      <c r="Z24" s="1"/>
-      <c r="AA24" s="1"/>
-      <c r="AB24" s="1"/>
+      <c r="A24" s="3"/>
+      <c r="B24" s="3"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
+      <c r="I24" s="3"/>
+      <c r="J24" s="3"/>
+      <c r="K24" s="3"/>
+      <c r="L24" s="3"/>
+      <c r="M24" s="3"/>
     </row>
     <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0"/>
-      <c r="B25" s="0"/>
-      <c r="D25" s="0"/>
-      <c r="E25" s="0"/>
-      <c r="F25" s="0"/>
-      <c r="G25" s="0"/>
-      <c r="H25" s="0"/>
-      <c r="I25" s="0"/>
-      <c r="J25" s="0"/>
-      <c r="K25" s="0"/>
-      <c r="L25" s="0"/>
-      <c r="M25" s="0"/>
-      <c r="N25" s="1"/>
-      <c r="O25" s="1"/>
-      <c r="P25" s="1"/>
-      <c r="Q25" s="1"/>
-      <c r="R25" s="1"/>
-      <c r="X25" s="1"/>
-      <c r="Y25" s="1"/>
-      <c r="Z25" s="1"/>
-      <c r="AA25" s="1"/>
-      <c r="AB25" s="1"/>
+      <c r="A25" s="3"/>
+      <c r="B25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3"/>
+      <c r="J25" s="3"/>
+      <c r="K25" s="3"/>
+      <c r="L25" s="3"/>
+      <c r="M25" s="3"/>
     </row>
     <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0"/>
-      <c r="B26" s="0"/>
-      <c r="D26" s="0"/>
-      <c r="E26" s="0"/>
-      <c r="F26" s="0"/>
-      <c r="G26" s="0"/>
-      <c r="H26" s="0"/>
-      <c r="I26" s="0"/>
-      <c r="J26" s="0"/>
-      <c r="K26" s="0"/>
-      <c r="L26" s="0"/>
-      <c r="M26" s="0"/>
-      <c r="N26" s="1"/>
-      <c r="O26" s="1"/>
-      <c r="P26" s="1"/>
-      <c r="Q26" s="1"/>
-      <c r="R26" s="1"/>
-      <c r="X26" s="1"/>
-      <c r="Y26" s="1"/>
-      <c r="Z26" s="1"/>
-      <c r="AA26" s="1"/>
-      <c r="AB26" s="1"/>
+      <c r="A26" s="3"/>
+      <c r="B26" s="3"/>
+      <c r="D26" s="3"/>
+      <c r="E26" s="3"/>
+      <c r="F26" s="3"/>
+      <c r="G26" s="3"/>
+      <c r="H26" s="3"/>
+      <c r="I26" s="3"/>
+      <c r="J26" s="3"/>
+      <c r="K26" s="3"/>
+      <c r="L26" s="3"/>
+      <c r="M26" s="3"/>
     </row>
     <row r="27" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="0"/>
-      <c r="B27" s="0"/>
-      <c r="D27" s="0"/>
-      <c r="E27" s="0"/>
-      <c r="F27" s="0"/>
-      <c r="G27" s="0"/>
-      <c r="H27" s="0"/>
-      <c r="I27" s="0"/>
-      <c r="J27" s="0"/>
-      <c r="K27" s="0"/>
-      <c r="L27" s="0"/>
-      <c r="M27" s="0"/>
-      <c r="N27" s="1"/>
-      <c r="O27" s="1"/>
-      <c r="P27" s="1"/>
-      <c r="Q27" s="1"/>
-      <c r="R27" s="1"/>
-      <c r="X27" s="1"/>
-      <c r="Y27" s="1"/>
-      <c r="Z27" s="1"/>
-      <c r="AA27" s="1"/>
-      <c r="AB27" s="1"/>
+      <c r="A27" s="3"/>
+      <c r="B27" s="3"/>
+      <c r="D27" s="3"/>
+      <c r="E27" s="3"/>
+      <c r="F27" s="3"/>
+      <c r="G27" s="3"/>
+      <c r="H27" s="3"/>
+      <c r="I27" s="3"/>
+      <c r="J27" s="3"/>
+      <c r="K27" s="3"/>
+      <c r="L27" s="3"/>
+      <c r="M27" s="3"/>
     </row>
     <row r="28" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="0"/>
-      <c r="B28" s="0"/>
-      <c r="D28" s="0"/>
-      <c r="E28" s="0"/>
-      <c r="F28" s="0"/>
-      <c r="G28" s="0"/>
-      <c r="H28" s="0"/>
-      <c r="I28" s="0"/>
-      <c r="J28" s="0"/>
-      <c r="K28" s="0"/>
-      <c r="L28" s="0"/>
-      <c r="M28" s="0"/>
-      <c r="N28" s="1"/>
-      <c r="O28" s="1"/>
-      <c r="P28" s="1"/>
-      <c r="Q28" s="1"/>
-      <c r="R28" s="1"/>
-      <c r="X28" s="1"/>
-      <c r="Y28" s="1"/>
-      <c r="Z28" s="1"/>
-      <c r="AA28" s="1"/>
-      <c r="AB28" s="1"/>
+      <c r="A28" s="3"/>
+      <c r="B28" s="3"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+      <c r="H28" s="3"/>
+      <c r="I28" s="3"/>
+      <c r="J28" s="3"/>
+      <c r="K28" s="3"/>
+      <c r="L28" s="3"/>
+      <c r="M28" s="3"/>
     </row>
     <row r="29" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="0"/>
-      <c r="B29" s="0"/>
-      <c r="D29" s="0"/>
-      <c r="E29" s="0"/>
-      <c r="F29" s="0"/>
-      <c r="G29" s="0"/>
-      <c r="H29" s="0"/>
-      <c r="I29" s="0"/>
-      <c r="J29" s="0"/>
-      <c r="K29" s="0"/>
-      <c r="L29" s="0"/>
-      <c r="M29" s="0"/>
-      <c r="N29" s="1"/>
-      <c r="O29" s="1"/>
-      <c r="P29" s="1"/>
-      <c r="Q29" s="1"/>
-      <c r="R29" s="1"/>
-      <c r="X29" s="1"/>
-      <c r="Y29" s="1"/>
-      <c r="Z29" s="1"/>
-      <c r="AA29" s="1"/>
-      <c r="AB29" s="1"/>
+      <c r="A29" s="3"/>
+      <c r="B29" s="3"/>
+      <c r="D29" s="3"/>
+      <c r="E29" s="3"/>
+      <c r="F29" s="3"/>
+      <c r="G29" s="3"/>
+      <c r="H29" s="3"/>
+      <c r="I29" s="3"/>
+      <c r="J29" s="3"/>
+      <c r="K29" s="3"/>
+      <c r="L29" s="3"/>
+      <c r="M29" s="3"/>
     </row>
     <row r="30" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="0"/>
-      <c r="B30" s="0"/>
-      <c r="D30" s="0"/>
-      <c r="E30" s="0"/>
-      <c r="F30" s="0"/>
-      <c r="G30" s="0"/>
-      <c r="H30" s="0"/>
-      <c r="I30" s="0"/>
-      <c r="J30" s="0"/>
-      <c r="K30" s="0"/>
-      <c r="L30" s="0"/>
-      <c r="M30" s="0"/>
-      <c r="N30" s="1"/>
-      <c r="O30" s="1"/>
-      <c r="P30" s="1"/>
-      <c r="Q30" s="1"/>
-      <c r="R30" s="1"/>
-      <c r="X30" s="1"/>
-      <c r="Y30" s="1"/>
-      <c r="Z30" s="1"/>
-      <c r="AA30" s="1"/>
-      <c r="AB30" s="1"/>
+      <c r="A30" s="3"/>
+      <c r="B30" s="3"/>
+      <c r="D30" s="3"/>
+      <c r="E30" s="3"/>
+      <c r="F30" s="3"/>
+      <c r="G30" s="3"/>
+      <c r="H30" s="3"/>
+      <c r="I30" s="3"/>
+      <c r="J30" s="3"/>
+      <c r="K30" s="3"/>
+      <c r="L30" s="3"/>
+      <c r="M30" s="3"/>
     </row>
     <row r="31" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="0"/>
-      <c r="B31" s="0"/>
-      <c r="D31" s="0"/>
-      <c r="E31" s="0"/>
-      <c r="F31" s="0"/>
-      <c r="G31" s="0"/>
-      <c r="H31" s="0"/>
-      <c r="I31" s="0"/>
-      <c r="J31" s="0"/>
-      <c r="K31" s="0"/>
-      <c r="L31" s="0"/>
-      <c r="M31" s="0"/>
-      <c r="N31" s="1"/>
-      <c r="O31" s="1"/>
-      <c r="P31" s="1"/>
-      <c r="Q31" s="1"/>
-      <c r="R31" s="1"/>
-      <c r="X31" s="1"/>
-      <c r="Y31" s="1"/>
-      <c r="Z31" s="1"/>
-      <c r="AA31" s="1"/>
-      <c r="AB31" s="1"/>
+      <c r="A31" s="3"/>
+      <c r="B31" s="3"/>
+      <c r="D31" s="3"/>
+      <c r="E31" s="3"/>
+      <c r="F31" s="3"/>
+      <c r="G31" s="3"/>
+      <c r="H31" s="3"/>
+      <c r="I31" s="3"/>
+      <c r="J31" s="3"/>
+      <c r="K31" s="3"/>
+      <c r="L31" s="3"/>
+      <c r="M31" s="3"/>
     </row>
     <row r="32" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="0"/>
-      <c r="B32" s="0"/>
-      <c r="D32" s="0"/>
-      <c r="E32" s="0"/>
-      <c r="F32" s="0"/>
-      <c r="G32" s="0"/>
-      <c r="H32" s="0"/>
-      <c r="I32" s="0"/>
-      <c r="J32" s="0"/>
-      <c r="K32" s="0"/>
-      <c r="L32" s="0"/>
-      <c r="M32" s="0"/>
-      <c r="N32" s="1"/>
-      <c r="O32" s="1"/>
-      <c r="P32" s="1"/>
-      <c r="Q32" s="1"/>
-      <c r="R32" s="1"/>
-      <c r="X32" s="1"/>
-      <c r="Y32" s="1"/>
-      <c r="Z32" s="1"/>
-      <c r="AA32" s="1"/>
-      <c r="AB32" s="1"/>
+      <c r="A32" s="3"/>
+      <c r="B32" s="3"/>
+      <c r="D32" s="3"/>
+      <c r="E32" s="3"/>
+      <c r="F32" s="3"/>
+      <c r="G32" s="3"/>
+      <c r="H32" s="3"/>
+      <c r="I32" s="3"/>
+      <c r="J32" s="3"/>
+      <c r="K32" s="3"/>
+      <c r="L32" s="3"/>
+      <c r="M32" s="3"/>
     </row>
     <row r="33" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="0"/>
-      <c r="B33" s="0"/>
-      <c r="D33" s="0"/>
-      <c r="E33" s="0"/>
-      <c r="F33" s="0"/>
-      <c r="G33" s="0"/>
-      <c r="H33" s="0"/>
-      <c r="I33" s="0"/>
-      <c r="J33" s="0"/>
-      <c r="K33" s="0"/>
-      <c r="L33" s="0"/>
-      <c r="M33" s="0"/>
-      <c r="N33" s="1"/>
-      <c r="O33" s="1"/>
-      <c r="P33" s="1"/>
-      <c r="Q33" s="1"/>
-      <c r="R33" s="1"/>
-      <c r="X33" s="1"/>
-      <c r="Y33" s="1"/>
-      <c r="Z33" s="1"/>
-      <c r="AA33" s="1"/>
-      <c r="AB33" s="1"/>
+      <c r="A33" s="3"/>
+      <c r="B33" s="3"/>
+      <c r="D33" s="3"/>
+      <c r="E33" s="3"/>
+      <c r="F33" s="3"/>
+      <c r="G33" s="3"/>
+      <c r="H33" s="3"/>
+      <c r="I33" s="3"/>
+      <c r="J33" s="3"/>
+      <c r="K33" s="3"/>
+      <c r="L33" s="3"/>
+      <c r="M33" s="3"/>
     </row>
     <row r="34" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="0"/>
-      <c r="B34" s="0"/>
-      <c r="D34" s="0"/>
-      <c r="E34" s="0"/>
-      <c r="F34" s="0"/>
-      <c r="G34" s="0"/>
-      <c r="H34" s="0"/>
-      <c r="I34" s="0"/>
-      <c r="J34" s="0"/>
-      <c r="K34" s="0"/>
-      <c r="L34" s="0"/>
-      <c r="M34" s="0"/>
-      <c r="N34" s="1"/>
-      <c r="O34" s="1"/>
-      <c r="P34" s="1"/>
-      <c r="Q34" s="1"/>
-      <c r="R34" s="1"/>
-      <c r="X34" s="1"/>
-      <c r="Y34" s="1"/>
-      <c r="Z34" s="1"/>
-      <c r="AA34" s="1"/>
-      <c r="AB34" s="1"/>
+      <c r="A34" s="3"/>
+      <c r="B34" s="3"/>
+      <c r="D34" s="3"/>
+      <c r="E34" s="3"/>
+      <c r="F34" s="3"/>
+      <c r="G34" s="3"/>
+      <c r="H34" s="3"/>
+      <c r="I34" s="3"/>
+      <c r="J34" s="3"/>
+      <c r="K34" s="3"/>
+      <c r="L34" s="3"/>
+      <c r="M34" s="3"/>
     </row>
     <row r="35" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="0"/>
-      <c r="B35" s="0"/>
-      <c r="D35" s="0"/>
-      <c r="E35" s="0"/>
-      <c r="F35" s="0"/>
-      <c r="G35" s="0"/>
-      <c r="H35" s="0"/>
-      <c r="I35" s="0"/>
-      <c r="J35" s="0"/>
-      <c r="K35" s="0"/>
-      <c r="L35" s="0"/>
-      <c r="M35" s="0"/>
-      <c r="N35" s="1"/>
-      <c r="O35" s="1"/>
-      <c r="P35" s="1"/>
-      <c r="Q35" s="1"/>
-      <c r="R35" s="1"/>
-      <c r="X35" s="1"/>
-      <c r="Y35" s="1"/>
-      <c r="Z35" s="1"/>
-      <c r="AA35" s="1"/>
-      <c r="AB35" s="1"/>
+      <c r="A35" s="3"/>
+      <c r="B35" s="3"/>
+      <c r="D35" s="3"/>
+      <c r="E35" s="3"/>
+      <c r="F35" s="3"/>
+      <c r="G35" s="3"/>
+      <c r="H35" s="3"/>
+      <c r="I35" s="3"/>
+      <c r="J35" s="3"/>
+      <c r="K35" s="3"/>
+      <c r="L35" s="3"/>
+      <c r="M35" s="3"/>
     </row>
     <row r="36" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="0"/>
-      <c r="B36" s="0"/>
-      <c r="D36" s="0"/>
-      <c r="E36" s="0"/>
-      <c r="F36" s="0"/>
-      <c r="G36" s="0"/>
-      <c r="H36" s="0"/>
-      <c r="I36" s="0"/>
-      <c r="J36" s="0"/>
-      <c r="K36" s="0"/>
-      <c r="L36" s="0"/>
-      <c r="M36" s="0"/>
-      <c r="N36" s="1"/>
-      <c r="O36" s="1"/>
-      <c r="P36" s="1"/>
-      <c r="Q36" s="1"/>
-      <c r="R36" s="1"/>
-      <c r="X36" s="1"/>
-      <c r="Y36" s="1"/>
-      <c r="Z36" s="1"/>
-      <c r="AA36" s="1"/>
-      <c r="AB36" s="1"/>
+      <c r="A36" s="3"/>
+      <c r="B36" s="3"/>
+      <c r="D36" s="3"/>
+      <c r="E36" s="3"/>
+      <c r="F36" s="3"/>
+      <c r="G36" s="3"/>
+      <c r="H36" s="3"/>
+      <c r="I36" s="3"/>
+      <c r="J36" s="3"/>
+      <c r="K36" s="3"/>
+      <c r="L36" s="3"/>
+      <c r="M36" s="3"/>
     </row>
     <row r="37" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="0"/>
-      <c r="B37" s="0"/>
-      <c r="D37" s="0"/>
-      <c r="E37" s="0"/>
-      <c r="F37" s="0"/>
-      <c r="G37" s="0"/>
-      <c r="H37" s="0"/>
-      <c r="I37" s="0"/>
-      <c r="J37" s="0"/>
-      <c r="K37" s="0"/>
-      <c r="L37" s="0"/>
-      <c r="M37" s="0"/>
-      <c r="N37" s="1"/>
-      <c r="O37" s="1"/>
-      <c r="P37" s="1"/>
-      <c r="Q37" s="1"/>
-      <c r="R37" s="1"/>
-      <c r="X37" s="1"/>
-      <c r="Y37" s="1"/>
-      <c r="Z37" s="1"/>
-      <c r="AA37" s="1"/>
-      <c r="AB37" s="1"/>
+      <c r="A37" s="3"/>
+      <c r="B37" s="3"/>
+      <c r="D37" s="3"/>
+      <c r="E37" s="3"/>
+      <c r="F37" s="3"/>
+      <c r="G37" s="3"/>
+      <c r="H37" s="3"/>
+      <c r="I37" s="3"/>
+      <c r="J37" s="3"/>
+      <c r="K37" s="3"/>
+      <c r="L37" s="3"/>
+      <c r="M37" s="3"/>
     </row>
     <row r="38" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="0"/>
-      <c r="B38" s="0"/>
-      <c r="D38" s="0"/>
-      <c r="E38" s="0"/>
-      <c r="F38" s="0"/>
-      <c r="G38" s="0"/>
-      <c r="H38" s="0"/>
-      <c r="I38" s="0"/>
-      <c r="J38" s="0"/>
-      <c r="K38" s="0"/>
-      <c r="L38" s="0"/>
-      <c r="M38" s="0"/>
-      <c r="N38" s="1"/>
-      <c r="O38" s="1"/>
-      <c r="P38" s="1"/>
-      <c r="Q38" s="1"/>
-      <c r="R38" s="1"/>
-      <c r="X38" s="1"/>
-      <c r="Y38" s="1"/>
-      <c r="Z38" s="1"/>
-      <c r="AA38" s="1"/>
-      <c r="AB38" s="1"/>
+      <c r="A38" s="3"/>
+      <c r="B38" s="3"/>
+      <c r="D38" s="3"/>
+      <c r="E38" s="3"/>
+      <c r="F38" s="3"/>
+      <c r="G38" s="3"/>
+      <c r="H38" s="3"/>
+      <c r="I38" s="3"/>
+      <c r="J38" s="3"/>
+      <c r="K38" s="3"/>
+      <c r="L38" s="3"/>
+      <c r="M38" s="3"/>
     </row>
     <row r="39" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="0"/>
-      <c r="B39" s="0"/>
-      <c r="D39" s="0"/>
-      <c r="E39" s="0"/>
-      <c r="F39" s="0"/>
-      <c r="G39" s="0"/>
-      <c r="H39" s="0"/>
-      <c r="I39" s="0"/>
-      <c r="J39" s="0"/>
-      <c r="K39" s="0"/>
-      <c r="L39" s="0"/>
-      <c r="M39" s="0"/>
-      <c r="N39" s="1"/>
-      <c r="O39" s="1"/>
-      <c r="P39" s="1"/>
-      <c r="Q39" s="1"/>
-      <c r="R39" s="1"/>
-      <c r="X39" s="1"/>
-      <c r="Y39" s="1"/>
-      <c r="Z39" s="1"/>
-      <c r="AA39" s="1"/>
-      <c r="AB39" s="1"/>
+      <c r="A39" s="3"/>
+      <c r="B39" s="3"/>
+      <c r="D39" s="3"/>
+      <c r="E39" s="3"/>
+      <c r="F39" s="3"/>
+      <c r="G39" s="3"/>
+      <c r="H39" s="3"/>
+      <c r="I39" s="3"/>
+      <c r="J39" s="3"/>
+      <c r="K39" s="3"/>
+      <c r="L39" s="3"/>
+      <c r="M39" s="3"/>
     </row>
     <row r="40" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="0"/>
-      <c r="B40" s="0"/>
-      <c r="D40" s="0"/>
-      <c r="E40" s="0"/>
-      <c r="F40" s="0"/>
-      <c r="G40" s="0"/>
-      <c r="H40" s="0"/>
-      <c r="I40" s="0"/>
-      <c r="J40" s="0"/>
-      <c r="K40" s="0"/>
-      <c r="L40" s="0"/>
-      <c r="M40" s="0"/>
-      <c r="N40" s="1"/>
-      <c r="O40" s="1"/>
-      <c r="P40" s="1"/>
-      <c r="Q40" s="1"/>
-      <c r="R40" s="1"/>
-      <c r="X40" s="1"/>
-      <c r="Y40" s="1"/>
-      <c r="Z40" s="1"/>
-      <c r="AA40" s="1"/>
-      <c r="AB40" s="1"/>
+      <c r="A40" s="3"/>
+      <c r="B40" s="3"/>
+      <c r="D40" s="3"/>
+      <c r="E40" s="3"/>
+      <c r="F40" s="3"/>
+      <c r="G40" s="3"/>
+      <c r="H40" s="3"/>
+      <c r="I40" s="3"/>
+      <c r="J40" s="3"/>
+      <c r="K40" s="3"/>
+      <c r="L40" s="3"/>
+      <c r="M40" s="3"/>
     </row>
     <row r="41" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="0"/>
-      <c r="B41" s="0"/>
-      <c r="D41" s="0"/>
-      <c r="E41" s="0"/>
-      <c r="F41" s="0"/>
-      <c r="G41" s="0"/>
-      <c r="H41" s="0"/>
-      <c r="I41" s="0"/>
-      <c r="J41" s="0"/>
-      <c r="K41" s="0"/>
-      <c r="L41" s="0"/>
-      <c r="M41" s="0"/>
-      <c r="N41" s="1"/>
-      <c r="O41" s="1"/>
-      <c r="P41" s="1"/>
-      <c r="Q41" s="1"/>
-      <c r="R41" s="1"/>
-      <c r="X41" s="1"/>
-      <c r="Y41" s="1"/>
-      <c r="Z41" s="1"/>
-      <c r="AA41" s="1"/>
-      <c r="AB41" s="1"/>
+      <c r="A41" s="3"/>
+      <c r="B41" s="3"/>
+      <c r="D41" s="3"/>
+      <c r="E41" s="3"/>
+      <c r="F41" s="3"/>
+      <c r="G41" s="3"/>
+      <c r="H41" s="3"/>
+      <c r="I41" s="3"/>
+      <c r="J41" s="3"/>
+      <c r="K41" s="3"/>
+      <c r="L41" s="3"/>
+      <c r="M41" s="3"/>
     </row>
     <row r="42" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="0"/>
-      <c r="B42" s="0"/>
-      <c r="D42" s="0"/>
-      <c r="E42" s="0"/>
-      <c r="F42" s="0"/>
-      <c r="G42" s="0"/>
-      <c r="H42" s="0"/>
-      <c r="I42" s="0"/>
-      <c r="J42" s="0"/>
-      <c r="K42" s="0"/>
-      <c r="L42" s="0"/>
-      <c r="M42" s="0"/>
-      <c r="N42" s="1"/>
-      <c r="O42" s="1"/>
-      <c r="P42" s="1"/>
-      <c r="Q42" s="1"/>
-      <c r="R42" s="1"/>
-      <c r="X42" s="1"/>
-      <c r="Y42" s="1"/>
-      <c r="Z42" s="1"/>
-      <c r="AA42" s="1"/>
-      <c r="AB42" s="1"/>
+      <c r="A42" s="3"/>
+      <c r="B42" s="3"/>
+      <c r="D42" s="3"/>
+      <c r="E42" s="3"/>
+      <c r="F42" s="3"/>
+      <c r="G42" s="3"/>
+      <c r="H42" s="3"/>
+      <c r="I42" s="3"/>
+      <c r="J42" s="3"/>
+      <c r="K42" s="3"/>
+      <c r="L42" s="3"/>
+      <c r="M42" s="3"/>
     </row>
     <row r="43" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="0"/>
-      <c r="B43" s="0"/>
-      <c r="D43" s="0"/>
-      <c r="E43" s="0"/>
-      <c r="F43" s="0"/>
-      <c r="G43" s="0"/>
-      <c r="H43" s="0"/>
-      <c r="I43" s="0"/>
-      <c r="J43" s="0"/>
-      <c r="K43" s="0"/>
-      <c r="L43" s="0"/>
-      <c r="M43" s="0"/>
-      <c r="N43" s="1"/>
-      <c r="O43" s="1"/>
-      <c r="P43" s="1"/>
-      <c r="Q43" s="1"/>
-      <c r="R43" s="1"/>
-      <c r="X43" s="1"/>
-      <c r="Y43" s="1"/>
-      <c r="Z43" s="1"/>
-      <c r="AA43" s="1"/>
-      <c r="AB43" s="1"/>
+      <c r="A43" s="3"/>
+      <c r="B43" s="3"/>
+      <c r="D43" s="3"/>
+      <c r="E43" s="3"/>
+      <c r="F43" s="3"/>
+      <c r="G43" s="3"/>
+      <c r="H43" s="3"/>
+      <c r="I43" s="3"/>
+      <c r="J43" s="3"/>
+      <c r="K43" s="3"/>
+      <c r="L43" s="3"/>
+      <c r="M43" s="3"/>
     </row>
     <row r="44" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="0"/>
-      <c r="B44" s="0"/>
-      <c r="D44" s="0"/>
-      <c r="E44" s="0"/>
-      <c r="F44" s="0"/>
-      <c r="G44" s="0"/>
-      <c r="H44" s="0"/>
-      <c r="I44" s="0"/>
-      <c r="J44" s="0"/>
-      <c r="K44" s="0"/>
-      <c r="L44" s="0"/>
-      <c r="M44" s="0"/>
-      <c r="N44" s="1"/>
-      <c r="O44" s="1"/>
-      <c r="P44" s="1"/>
-      <c r="Q44" s="1"/>
-      <c r="R44" s="1"/>
-      <c r="X44" s="1"/>
-      <c r="Y44" s="1"/>
-      <c r="Z44" s="1"/>
-      <c r="AA44" s="1"/>
-      <c r="AB44" s="1"/>
+      <c r="A44" s="3"/>
+      <c r="B44" s="3"/>
+      <c r="D44" s="3"/>
+      <c r="E44" s="3"/>
+      <c r="F44" s="3"/>
+      <c r="G44" s="3"/>
+      <c r="H44" s="3"/>
+      <c r="I44" s="3"/>
+      <c r="J44" s="3"/>
+      <c r="K44" s="3"/>
+      <c r="L44" s="3"/>
+      <c r="M44" s="3"/>
     </row>
     <row r="45" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="0"/>
-      <c r="B45" s="0"/>
-      <c r="D45" s="0"/>
-      <c r="E45" s="0"/>
-      <c r="F45" s="0"/>
-      <c r="G45" s="0"/>
-      <c r="H45" s="0"/>
-      <c r="I45" s="0"/>
-      <c r="J45" s="0"/>
-      <c r="K45" s="0"/>
-      <c r="L45" s="0"/>
-      <c r="M45" s="0"/>
-      <c r="N45" s="1"/>
-      <c r="O45" s="1"/>
-      <c r="P45" s="1"/>
-      <c r="Q45" s="1"/>
-      <c r="R45" s="1"/>
-      <c r="X45" s="1"/>
-      <c r="Y45" s="1"/>
-      <c r="Z45" s="1"/>
-      <c r="AA45" s="1"/>
-      <c r="AB45" s="1"/>
+      <c r="A45" s="3"/>
+      <c r="B45" s="3"/>
+      <c r="D45" s="3"/>
+      <c r="E45" s="3"/>
+      <c r="F45" s="3"/>
+      <c r="G45" s="3"/>
+      <c r="H45" s="3"/>
+      <c r="I45" s="3"/>
+      <c r="J45" s="3"/>
+      <c r="K45" s="3"/>
+      <c r="L45" s="3"/>
+      <c r="M45" s="3"/>
     </row>
     <row r="46" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="0"/>
-      <c r="B46" s="0"/>
-      <c r="D46" s="0"/>
-      <c r="E46" s="0"/>
-      <c r="F46" s="0"/>
-      <c r="G46" s="0"/>
-      <c r="H46" s="0"/>
-      <c r="I46" s="0"/>
-      <c r="J46" s="0"/>
-      <c r="K46" s="0"/>
-      <c r="L46" s="0"/>
-      <c r="M46" s="0"/>
-      <c r="N46" s="1"/>
-      <c r="O46" s="1"/>
-      <c r="P46" s="1"/>
-      <c r="Q46" s="1"/>
-      <c r="R46" s="1"/>
-      <c r="X46" s="1"/>
-      <c r="Y46" s="1"/>
-      <c r="Z46" s="1"/>
-      <c r="AA46" s="1"/>
-      <c r="AB46" s="1"/>
+      <c r="A46" s="3"/>
+      <c r="B46" s="3"/>
+      <c r="D46" s="3"/>
+      <c r="E46" s="3"/>
+      <c r="F46" s="3"/>
+      <c r="G46" s="3"/>
+      <c r="H46" s="3"/>
+      <c r="I46" s="3"/>
+      <c r="J46" s="3"/>
+      <c r="K46" s="3"/>
+      <c r="L46" s="3"/>
+      <c r="M46" s="3"/>
     </row>
     <row r="47" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="0"/>
-      <c r="B47" s="0"/>
-      <c r="D47" s="0"/>
-      <c r="E47" s="0"/>
-      <c r="F47" s="0"/>
-      <c r="G47" s="0"/>
-      <c r="H47" s="0"/>
-      <c r="I47" s="0"/>
-      <c r="J47" s="0"/>
-      <c r="K47" s="0"/>
-      <c r="L47" s="0"/>
-      <c r="M47" s="0"/>
-      <c r="N47" s="1"/>
-      <c r="O47" s="1"/>
-      <c r="P47" s="1"/>
-      <c r="Q47" s="1"/>
-      <c r="R47" s="1"/>
-      <c r="X47" s="1"/>
-      <c r="Y47" s="1"/>
-      <c r="Z47" s="1"/>
-      <c r="AA47" s="1"/>
-      <c r="AB47" s="1"/>
+      <c r="A47" s="3"/>
+      <c r="B47" s="3"/>
+      <c r="D47" s="3"/>
+      <c r="E47" s="3"/>
+      <c r="F47" s="3"/>
+      <c r="G47" s="3"/>
+      <c r="H47" s="3"/>
+      <c r="I47" s="3"/>
+      <c r="J47" s="3"/>
+      <c r="K47" s="3"/>
+      <c r="L47" s="3"/>
+      <c r="M47" s="3"/>
     </row>
     <row r="48" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="0"/>
-      <c r="B48" s="0"/>
-      <c r="D48" s="0"/>
-      <c r="E48" s="0"/>
-      <c r="F48" s="0"/>
-      <c r="G48" s="0"/>
-      <c r="H48" s="0"/>
-      <c r="I48" s="0"/>
-      <c r="J48" s="0"/>
-      <c r="K48" s="0"/>
-      <c r="L48" s="0"/>
-      <c r="M48" s="0"/>
-      <c r="N48" s="1"/>
-      <c r="O48" s="1"/>
-      <c r="P48" s="1"/>
-      <c r="Q48" s="1"/>
-      <c r="R48" s="1"/>
-      <c r="X48" s="1"/>
-      <c r="Y48" s="1"/>
-      <c r="Z48" s="1"/>
-      <c r="AA48" s="1"/>
-      <c r="AB48" s="1"/>
+      <c r="A48" s="3"/>
+      <c r="B48" s="3"/>
+      <c r="D48" s="3"/>
+      <c r="E48" s="3"/>
+      <c r="F48" s="3"/>
+      <c r="G48" s="3"/>
+      <c r="H48" s="3"/>
+      <c r="I48" s="3"/>
+      <c r="J48" s="3"/>
+      <c r="K48" s="3"/>
+      <c r="L48" s="3"/>
+      <c r="M48" s="3"/>
     </row>
     <row r="49" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="0"/>
-      <c r="B49" s="0"/>
-      <c r="D49" s="0"/>
-      <c r="E49" s="0"/>
-      <c r="F49" s="0"/>
-      <c r="G49" s="0"/>
-      <c r="H49" s="0"/>
-      <c r="I49" s="0"/>
-      <c r="J49" s="0"/>
-      <c r="K49" s="0"/>
-      <c r="L49" s="0"/>
-      <c r="M49" s="0"/>
-      <c r="N49" s="1"/>
-      <c r="O49" s="1"/>
-      <c r="P49" s="1"/>
-      <c r="Q49" s="1"/>
-      <c r="R49" s="1"/>
-      <c r="X49" s="1"/>
-      <c r="Y49" s="1"/>
-      <c r="Z49" s="1"/>
-      <c r="AA49" s="1"/>
-      <c r="AB49" s="1"/>
+      <c r="A49" s="3"/>
+      <c r="B49" s="3"/>
+      <c r="D49" s="3"/>
+      <c r="E49" s="3"/>
+      <c r="F49" s="3"/>
+      <c r="G49" s="3"/>
+      <c r="H49" s="3"/>
+      <c r="I49" s="3"/>
+      <c r="J49" s="3"/>
+      <c r="K49" s="3"/>
+      <c r="L49" s="3"/>
+      <c r="M49" s="3"/>
     </row>
     <row r="50" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="0"/>
-      <c r="B50" s="0"/>
-      <c r="D50" s="0"/>
-      <c r="E50" s="0"/>
-      <c r="F50" s="0"/>
-      <c r="G50" s="0"/>
-      <c r="H50" s="0"/>
-      <c r="I50" s="0"/>
-      <c r="J50" s="0"/>
-      <c r="K50" s="0"/>
-      <c r="L50" s="0"/>
-      <c r="M50" s="0"/>
-      <c r="N50" s="1"/>
-      <c r="O50" s="1"/>
-      <c r="P50" s="1"/>
-      <c r="Q50" s="1"/>
-      <c r="R50" s="1"/>
-      <c r="X50" s="1"/>
-      <c r="Y50" s="1"/>
-      <c r="Z50" s="1"/>
-      <c r="AA50" s="1"/>
-      <c r="AB50" s="1"/>
+      <c r="A50" s="3"/>
+      <c r="B50" s="3"/>
+      <c r="D50" s="3"/>
+      <c r="E50" s="3"/>
+      <c r="F50" s="3"/>
+      <c r="G50" s="3"/>
+      <c r="H50" s="3"/>
+      <c r="I50" s="3"/>
+      <c r="J50" s="3"/>
+      <c r="K50" s="3"/>
+      <c r="L50" s="3"/>
+      <c r="M50" s="3"/>
     </row>
     <row r="51" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="0"/>
-      <c r="B51" s="0"/>
-      <c r="D51" s="0"/>
-      <c r="E51" s="0"/>
-      <c r="F51" s="0"/>
-      <c r="G51" s="0"/>
-      <c r="H51" s="0"/>
-      <c r="I51" s="0"/>
-      <c r="J51" s="0"/>
-      <c r="K51" s="0"/>
-      <c r="L51" s="0"/>
-      <c r="M51" s="0"/>
-      <c r="N51" s="1"/>
-      <c r="O51" s="1"/>
-      <c r="P51" s="1"/>
-      <c r="Q51" s="1"/>
-      <c r="R51" s="1"/>
-      <c r="X51" s="1"/>
-      <c r="Y51" s="1"/>
-      <c r="Z51" s="1"/>
-      <c r="AA51" s="1"/>
-      <c r="AB51" s="1"/>
+      <c r="A51" s="3"/>
+      <c r="B51" s="3"/>
+      <c r="D51" s="3"/>
+      <c r="E51" s="3"/>
+      <c r="F51" s="3"/>
+      <c r="G51" s="3"/>
+      <c r="H51" s="3"/>
+      <c r="I51" s="3"/>
+      <c r="J51" s="3"/>
+      <c r="K51" s="3"/>
+      <c r="L51" s="3"/>
+      <c r="M51" s="3"/>
     </row>
     <row r="52" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="0"/>
-      <c r="B52" s="0"/>
-      <c r="D52" s="0"/>
-      <c r="E52" s="0"/>
-      <c r="F52" s="0"/>
-      <c r="G52" s="0"/>
-      <c r="H52" s="0"/>
-      <c r="I52" s="0"/>
-      <c r="J52" s="0"/>
-      <c r="K52" s="0"/>
-      <c r="L52" s="0"/>
-      <c r="M52" s="0"/>
-      <c r="N52" s="1"/>
-      <c r="O52" s="1"/>
-      <c r="P52" s="1"/>
-      <c r="Q52" s="1"/>
-      <c r="R52" s="1"/>
-      <c r="X52" s="1"/>
-      <c r="Y52" s="1"/>
-      <c r="Z52" s="1"/>
-      <c r="AA52" s="1"/>
-      <c r="AB52" s="1"/>
+      <c r="A52" s="3"/>
+      <c r="B52" s="3"/>
+      <c r="D52" s="3"/>
+      <c r="E52" s="3"/>
+      <c r="F52" s="3"/>
+      <c r="G52" s="3"/>
+      <c r="H52" s="3"/>
+      <c r="I52" s="3"/>
+      <c r="J52" s="3"/>
+      <c r="K52" s="3"/>
+      <c r="L52" s="3"/>
+      <c r="M52" s="3"/>
     </row>
     <row r="53" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="0"/>
-      <c r="B53" s="0"/>
-      <c r="D53" s="0"/>
-      <c r="E53" s="0"/>
-      <c r="F53" s="0"/>
-      <c r="G53" s="0"/>
-      <c r="H53" s="0"/>
-      <c r="I53" s="0"/>
-      <c r="J53" s="0"/>
-      <c r="K53" s="0"/>
-      <c r="L53" s="0"/>
-      <c r="M53" s="0"/>
-      <c r="N53" s="1"/>
-      <c r="O53" s="1"/>
-      <c r="P53" s="1"/>
-      <c r="Q53" s="1"/>
-      <c r="R53" s="1"/>
-      <c r="X53" s="1"/>
-      <c r="Y53" s="1"/>
-      <c r="Z53" s="1"/>
-      <c r="AA53" s="1"/>
-      <c r="AB53" s="1"/>
+      <c r="A53" s="3"/>
+      <c r="B53" s="3"/>
+      <c r="D53" s="3"/>
+      <c r="E53" s="3"/>
+      <c r="F53" s="3"/>
+      <c r="G53" s="3"/>
+      <c r="H53" s="3"/>
+      <c r="I53" s="3"/>
+      <c r="J53" s="3"/>
+      <c r="K53" s="3"/>
+      <c r="L53" s="3"/>
+      <c r="M53" s="3"/>
     </row>
     <row r="54" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="0"/>
-      <c r="B54" s="0"/>
-      <c r="D54" s="0"/>
-      <c r="E54" s="0"/>
-      <c r="F54" s="0"/>
-      <c r="G54" s="0"/>
-      <c r="H54" s="0"/>
-      <c r="I54" s="0"/>
-      <c r="J54" s="0"/>
-      <c r="K54" s="0"/>
-      <c r="L54" s="0"/>
-      <c r="M54" s="0"/>
-      <c r="N54" s="1"/>
-      <c r="O54" s="1"/>
-      <c r="P54" s="1"/>
-      <c r="Q54" s="1"/>
-      <c r="R54" s="1"/>
-      <c r="X54" s="1"/>
-      <c r="Y54" s="1"/>
-      <c r="Z54" s="1"/>
-      <c r="AA54" s="1"/>
-      <c r="AB54" s="1"/>
+      <c r="A54" s="3"/>
+      <c r="B54" s="3"/>
+      <c r="D54" s="3"/>
+      <c r="E54" s="3"/>
+      <c r="F54" s="3"/>
+      <c r="G54" s="3"/>
+      <c r="H54" s="3"/>
+      <c r="I54" s="3"/>
+      <c r="J54" s="3"/>
+      <c r="K54" s="3"/>
+      <c r="L54" s="3"/>
+      <c r="M54" s="3"/>
     </row>
     <row r="55" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="0"/>
-      <c r="B55" s="0"/>
-      <c r="D55" s="0"/>
-      <c r="E55" s="0"/>
-      <c r="F55" s="0"/>
-      <c r="G55" s="0"/>
-      <c r="H55" s="0"/>
-      <c r="I55" s="0"/>
-      <c r="J55" s="0"/>
-      <c r="K55" s="0"/>
-      <c r="L55" s="0"/>
-      <c r="M55" s="0"/>
-      <c r="N55" s="1"/>
-      <c r="O55" s="1"/>
-      <c r="P55" s="1"/>
-      <c r="Q55" s="1"/>
-      <c r="R55" s="1"/>
-      <c r="X55" s="1"/>
-      <c r="Y55" s="1"/>
-      <c r="Z55" s="1"/>
-      <c r="AA55" s="1"/>
-      <c r="AB55" s="1"/>
+      <c r="A55" s="3"/>
+      <c r="B55" s="3"/>
+      <c r="D55" s="3"/>
+      <c r="E55" s="3"/>
+      <c r="F55" s="3"/>
+      <c r="G55" s="3"/>
+      <c r="H55" s="3"/>
+      <c r="I55" s="3"/>
+      <c r="J55" s="3"/>
+      <c r="K55" s="3"/>
+      <c r="L55" s="3"/>
+      <c r="M55" s="3"/>
     </row>
     <row r="56" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="0"/>
-      <c r="B56" s="0"/>
-      <c r="D56" s="0"/>
-      <c r="E56" s="0"/>
-      <c r="F56" s="0"/>
-      <c r="G56" s="0"/>
-      <c r="H56" s="0"/>
-      <c r="I56" s="0"/>
-      <c r="J56" s="0"/>
-      <c r="K56" s="0"/>
-      <c r="L56" s="0"/>
-      <c r="M56" s="0"/>
-      <c r="N56" s="1"/>
-      <c r="O56" s="1"/>
-      <c r="P56" s="1"/>
-      <c r="Q56" s="1"/>
-      <c r="R56" s="1"/>
-      <c r="X56" s="1"/>
-      <c r="Y56" s="1"/>
-      <c r="Z56" s="1"/>
-      <c r="AA56" s="1"/>
-      <c r="AB56" s="1"/>
+      <c r="A56" s="3"/>
+      <c r="B56" s="3"/>
+      <c r="D56" s="3"/>
+      <c r="E56" s="3"/>
+      <c r="F56" s="3"/>
+      <c r="G56" s="3"/>
+      <c r="H56" s="3"/>
+      <c r="I56" s="3"/>
+      <c r="J56" s="3"/>
+      <c r="K56" s="3"/>
+      <c r="L56" s="3"/>
+      <c r="M56" s="3"/>
     </row>
     <row r="57" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="0"/>
-      <c r="B57" s="0"/>
-      <c r="D57" s="0"/>
-      <c r="E57" s="0"/>
-      <c r="F57" s="0"/>
-      <c r="G57" s="0"/>
-      <c r="H57" s="0"/>
-      <c r="I57" s="0"/>
-      <c r="J57" s="0"/>
-      <c r="K57" s="0"/>
-      <c r="L57" s="0"/>
-      <c r="M57" s="0"/>
-      <c r="N57" s="1"/>
-      <c r="O57" s="1"/>
-      <c r="P57" s="1"/>
-      <c r="Q57" s="1"/>
-      <c r="R57" s="1"/>
-      <c r="X57" s="1"/>
-      <c r="Y57" s="1"/>
-      <c r="Z57" s="1"/>
-      <c r="AA57" s="1"/>
-      <c r="AB57" s="1"/>
+      <c r="A57" s="3"/>
+      <c r="B57" s="3"/>
+      <c r="D57" s="3"/>
+      <c r="E57" s="3"/>
+      <c r="F57" s="3"/>
+      <c r="G57" s="3"/>
+      <c r="H57" s="3"/>
+      <c r="I57" s="3"/>
+      <c r="J57" s="3"/>
+      <c r="K57" s="3"/>
+      <c r="L57" s="3"/>
+      <c r="M57" s="3"/>
     </row>
     <row r="58" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="0"/>
-      <c r="B58" s="0"/>
-      <c r="D58" s="0"/>
-      <c r="E58" s="0"/>
-      <c r="F58" s="0"/>
-      <c r="G58" s="0"/>
-      <c r="H58" s="0"/>
-      <c r="I58" s="0"/>
-      <c r="J58" s="0"/>
-      <c r="K58" s="0"/>
-      <c r="L58" s="0"/>
-      <c r="M58" s="0"/>
-      <c r="N58" s="1"/>
-      <c r="O58" s="1"/>
-      <c r="P58" s="1"/>
-      <c r="Q58" s="1"/>
-      <c r="R58" s="1"/>
-      <c r="X58" s="1"/>
-      <c r="Y58" s="1"/>
-      <c r="Z58" s="1"/>
-      <c r="AA58" s="1"/>
-      <c r="AB58" s="1"/>
+      <c r="A58" s="3"/>
+      <c r="B58" s="3"/>
+      <c r="D58" s="3"/>
+      <c r="E58" s="3"/>
+      <c r="F58" s="3"/>
+      <c r="G58" s="3"/>
+      <c r="H58" s="3"/>
+      <c r="I58" s="3"/>
+      <c r="J58" s="3"/>
+      <c r="K58" s="3"/>
+      <c r="L58" s="3"/>
+      <c r="M58" s="3"/>
     </row>
     <row r="59" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="0"/>
-      <c r="B59" s="0"/>
-      <c r="D59" s="0"/>
-      <c r="E59" s="0"/>
-      <c r="F59" s="0"/>
-      <c r="G59" s="0"/>
-      <c r="H59" s="0"/>
-      <c r="I59" s="0"/>
-      <c r="J59" s="0"/>
-      <c r="K59" s="0"/>
-      <c r="L59" s="0"/>
-      <c r="M59" s="0"/>
-      <c r="N59" s="1"/>
-      <c r="O59" s="1"/>
-      <c r="P59" s="1"/>
-      <c r="Q59" s="1"/>
-      <c r="R59" s="1"/>
-      <c r="X59" s="1"/>
-      <c r="Y59" s="1"/>
-      <c r="Z59" s="1"/>
-      <c r="AA59" s="1"/>
-      <c r="AB59" s="1"/>
+      <c r="A59" s="3"/>
+      <c r="B59" s="3"/>
+      <c r="D59" s="3"/>
+      <c r="E59" s="3"/>
+      <c r="F59" s="3"/>
+      <c r="G59" s="3"/>
+      <c r="H59" s="3"/>
+      <c r="I59" s="3"/>
+      <c r="J59" s="3"/>
+      <c r="K59" s="3"/>
+      <c r="L59" s="3"/>
+      <c r="M59" s="3"/>
     </row>
     <row r="60" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="0"/>
-      <c r="B60" s="0"/>
-      <c r="D60" s="0"/>
-      <c r="E60" s="0"/>
-      <c r="F60" s="0"/>
-      <c r="G60" s="0"/>
-      <c r="H60" s="0"/>
-      <c r="I60" s="0"/>
-      <c r="J60" s="0"/>
-      <c r="K60" s="0"/>
-      <c r="L60" s="0"/>
-      <c r="M60" s="0"/>
-      <c r="N60" s="1"/>
-      <c r="O60" s="1"/>
-      <c r="P60" s="1"/>
-      <c r="Q60" s="1"/>
-      <c r="R60" s="1"/>
-      <c r="X60" s="1"/>
-      <c r="Y60" s="1"/>
-      <c r="Z60" s="1"/>
-      <c r="AA60" s="1"/>
-      <c r="AB60" s="1"/>
+      <c r="A60" s="3"/>
+      <c r="B60" s="3"/>
+      <c r="D60" s="3"/>
+      <c r="E60" s="3"/>
+      <c r="F60" s="3"/>
+      <c r="G60" s="3"/>
+      <c r="H60" s="3"/>
+      <c r="I60" s="3"/>
+      <c r="J60" s="3"/>
+      <c r="K60" s="3"/>
+      <c r="L60" s="3"/>
+      <c r="M60" s="3"/>
     </row>
     <row r="61" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="0"/>
-      <c r="B61" s="0"/>
-      <c r="D61" s="0"/>
-      <c r="E61" s="0"/>
-      <c r="F61" s="0"/>
-      <c r="G61" s="0"/>
-      <c r="H61" s="0"/>
-      <c r="I61" s="0"/>
-      <c r="J61" s="0"/>
-      <c r="K61" s="0"/>
-      <c r="L61" s="0"/>
-      <c r="M61" s="0"/>
-      <c r="N61" s="1"/>
-      <c r="O61" s="1"/>
-      <c r="P61" s="1"/>
-      <c r="Q61" s="1"/>
-      <c r="R61" s="1"/>
-      <c r="X61" s="1"/>
-      <c r="Y61" s="1"/>
-      <c r="Z61" s="1"/>
-      <c r="AA61" s="1"/>
-      <c r="AB61" s="1"/>
+      <c r="A61" s="3"/>
+      <c r="B61" s="3"/>
+      <c r="D61" s="3"/>
+      <c r="E61" s="3"/>
+      <c r="F61" s="3"/>
+      <c r="G61" s="3"/>
+      <c r="H61" s="3"/>
+      <c r="I61" s="3"/>
+      <c r="J61" s="3"/>
+      <c r="K61" s="3"/>
+      <c r="L61" s="3"/>
+      <c r="M61" s="3"/>
     </row>
     <row r="62" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="0"/>
-      <c r="B62" s="0"/>
-      <c r="D62" s="0"/>
-      <c r="E62" s="0"/>
-      <c r="F62" s="0"/>
-      <c r="G62" s="0"/>
-      <c r="H62" s="0"/>
-      <c r="I62" s="0"/>
-      <c r="J62" s="0"/>
-      <c r="K62" s="0"/>
-      <c r="L62" s="0"/>
-      <c r="M62" s="0"/>
-      <c r="N62" s="1"/>
-      <c r="O62" s="1"/>
-      <c r="P62" s="1"/>
-      <c r="Q62" s="1"/>
-      <c r="R62" s="1"/>
-      <c r="X62" s="1"/>
-      <c r="Y62" s="1"/>
-      <c r="Z62" s="1"/>
-      <c r="AA62" s="1"/>
-      <c r="AB62" s="1"/>
+      <c r="A62" s="3"/>
+      <c r="B62" s="3"/>
+      <c r="D62" s="3"/>
+      <c r="E62" s="3"/>
+      <c r="F62" s="3"/>
+      <c r="G62" s="3"/>
+      <c r="H62" s="3"/>
+      <c r="I62" s="3"/>
+      <c r="J62" s="3"/>
+      <c r="K62" s="3"/>
+      <c r="L62" s="3"/>
+      <c r="M62" s="3"/>
     </row>
     <row r="63" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="0"/>
-      <c r="B63" s="0"/>
-      <c r="D63" s="0"/>
-      <c r="E63" s="0"/>
-      <c r="F63" s="0"/>
-      <c r="G63" s="0"/>
-      <c r="H63" s="0"/>
-      <c r="I63" s="0"/>
-      <c r="J63" s="0"/>
-      <c r="K63" s="0"/>
-      <c r="L63" s="0"/>
-      <c r="M63" s="0"/>
-      <c r="N63" s="1"/>
-      <c r="O63" s="1"/>
-      <c r="P63" s="1"/>
-      <c r="Q63" s="1"/>
-      <c r="R63" s="1"/>
-      <c r="X63" s="1"/>
-      <c r="Y63" s="1"/>
-      <c r="Z63" s="1"/>
-      <c r="AA63" s="1"/>
-      <c r="AB63" s="1"/>
+      <c r="A63" s="3"/>
+      <c r="B63" s="3"/>
+      <c r="D63" s="3"/>
+      <c r="E63" s="3"/>
+      <c r="F63" s="3"/>
+      <c r="G63" s="3"/>
+      <c r="H63" s="3"/>
+      <c r="I63" s="3"/>
+      <c r="J63" s="3"/>
+      <c r="K63" s="3"/>
+      <c r="L63" s="3"/>
+      <c r="M63" s="3"/>
     </row>
     <row r="64" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="0"/>
-      <c r="B64" s="0"/>
-      <c r="D64" s="0"/>
-      <c r="E64" s="0"/>
-      <c r="F64" s="0"/>
-      <c r="G64" s="0"/>
-      <c r="H64" s="0"/>
-      <c r="I64" s="0"/>
-      <c r="J64" s="0"/>
-      <c r="K64" s="0"/>
-      <c r="L64" s="0"/>
-      <c r="M64" s="0"/>
-      <c r="N64" s="1"/>
-      <c r="O64" s="1"/>
-      <c r="P64" s="1"/>
-      <c r="Q64" s="1"/>
-      <c r="R64" s="1"/>
-      <c r="X64" s="1"/>
-      <c r="Y64" s="1"/>
-      <c r="Z64" s="1"/>
-      <c r="AA64" s="1"/>
-      <c r="AB64" s="1"/>
+      <c r="A64" s="3"/>
+      <c r="B64" s="3"/>
+      <c r="D64" s="3"/>
+      <c r="E64" s="3"/>
+      <c r="F64" s="3"/>
+      <c r="G64" s="3"/>
+      <c r="H64" s="3"/>
+      <c r="I64" s="3"/>
+      <c r="J64" s="3"/>
+      <c r="K64" s="3"/>
+      <c r="L64" s="3"/>
+      <c r="M64" s="3"/>
     </row>
     <row r="65" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="0"/>
-      <c r="B65" s="0"/>
-      <c r="D65" s="0"/>
-      <c r="E65" s="0"/>
-      <c r="F65" s="0"/>
-      <c r="G65" s="0"/>
-      <c r="H65" s="0"/>
-      <c r="I65" s="0"/>
-      <c r="J65" s="0"/>
-      <c r="K65" s="0"/>
-      <c r="L65" s="0"/>
-      <c r="M65" s="0"/>
-      <c r="N65" s="1"/>
-      <c r="O65" s="1"/>
-      <c r="P65" s="1"/>
-      <c r="Q65" s="1"/>
-      <c r="R65" s="1"/>
-      <c r="X65" s="1"/>
-      <c r="Y65" s="1"/>
-      <c r="Z65" s="1"/>
-      <c r="AA65" s="1"/>
-      <c r="AB65" s="1"/>
+      <c r="A65" s="3"/>
+      <c r="B65" s="3"/>
+      <c r="D65" s="3"/>
+      <c r="E65" s="3"/>
+      <c r="F65" s="3"/>
+      <c r="G65" s="3"/>
+      <c r="H65" s="3"/>
+      <c r="I65" s="3"/>
+      <c r="J65" s="3"/>
+      <c r="K65" s="3"/>
+      <c r="L65" s="3"/>
+      <c r="M65" s="3"/>
     </row>
     <row r="66" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="0"/>
-      <c r="B66" s="0"/>
-      <c r="D66" s="0"/>
-      <c r="E66" s="0"/>
-      <c r="F66" s="0"/>
-      <c r="G66" s="0"/>
-      <c r="H66" s="0"/>
-      <c r="I66" s="0"/>
-      <c r="J66" s="0"/>
-      <c r="K66" s="0"/>
-      <c r="L66" s="0"/>
-      <c r="M66" s="0"/>
-      <c r="N66" s="1"/>
-      <c r="O66" s="1"/>
-      <c r="P66" s="1"/>
-      <c r="Q66" s="1"/>
-      <c r="R66" s="1"/>
-      <c r="X66" s="1"/>
-      <c r="Y66" s="1"/>
-      <c r="Z66" s="1"/>
-      <c r="AA66" s="1"/>
-      <c r="AB66" s="1"/>
+      <c r="A66" s="3"/>
+      <c r="B66" s="3"/>
+      <c r="D66" s="3"/>
+      <c r="E66" s="3"/>
+      <c r="F66" s="3"/>
+      <c r="G66" s="3"/>
+      <c r="H66" s="3"/>
+      <c r="I66" s="3"/>
+      <c r="J66" s="3"/>
+      <c r="K66" s="3"/>
+      <c r="L66" s="3"/>
+      <c r="M66" s="3"/>
     </row>
     <row r="67" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A67" s="0"/>
-      <c r="B67" s="0"/>
-      <c r="D67" s="0"/>
-      <c r="E67" s="0"/>
-      <c r="F67" s="0"/>
-      <c r="G67" s="0"/>
-      <c r="H67" s="0"/>
-      <c r="I67" s="0"/>
-      <c r="J67" s="0"/>
-      <c r="K67" s="0"/>
-      <c r="L67" s="0"/>
-      <c r="M67" s="0"/>
-      <c r="N67" s="1"/>
-      <c r="O67" s="1"/>
-      <c r="P67" s="1"/>
-      <c r="Q67" s="1"/>
-      <c r="R67" s="1"/>
-      <c r="X67" s="1"/>
-      <c r="Y67" s="1"/>
-      <c r="Z67" s="1"/>
-      <c r="AA67" s="1"/>
-      <c r="AB67" s="1"/>
+      <c r="A67" s="3"/>
+      <c r="B67" s="3"/>
+      <c r="D67" s="3"/>
+      <c r="E67" s="3"/>
+      <c r="F67" s="3"/>
+      <c r="G67" s="3"/>
+      <c r="H67" s="3"/>
+      <c r="I67" s="3"/>
+      <c r="J67" s="3"/>
+      <c r="K67" s="3"/>
+      <c r="L67" s="3"/>
+      <c r="M67" s="3"/>
     </row>
     <row r="68" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A68" s="0"/>
-      <c r="B68" s="0"/>
-      <c r="D68" s="0"/>
-      <c r="E68" s="0"/>
-      <c r="F68" s="0"/>
-      <c r="G68" s="0"/>
-      <c r="H68" s="0"/>
-      <c r="I68" s="0"/>
-      <c r="J68" s="0"/>
-      <c r="K68" s="0"/>
-      <c r="L68" s="0"/>
-      <c r="M68" s="0"/>
-      <c r="N68" s="1"/>
-      <c r="O68" s="1"/>
-      <c r="P68" s="1"/>
-      <c r="Q68" s="1"/>
-      <c r="R68" s="1"/>
-      <c r="X68" s="1"/>
-      <c r="Y68" s="1"/>
-      <c r="Z68" s="1"/>
-      <c r="AA68" s="1"/>
-      <c r="AB68" s="1"/>
+      <c r="A68" s="3"/>
+      <c r="B68" s="3"/>
+      <c r="D68" s="3"/>
+      <c r="E68" s="3"/>
+      <c r="F68" s="3"/>
+      <c r="G68" s="3"/>
+      <c r="H68" s="3"/>
+      <c r="I68" s="3"/>
+      <c r="J68" s="3"/>
+      <c r="K68" s="3"/>
+      <c r="L68" s="3"/>
+      <c r="M68" s="3"/>
     </row>
     <row r="69" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="0"/>
-      <c r="B69" s="0"/>
-      <c r="D69" s="0"/>
-      <c r="E69" s="0"/>
-      <c r="F69" s="0"/>
-      <c r="G69" s="0"/>
-      <c r="H69" s="0"/>
-      <c r="I69" s="0"/>
-      <c r="J69" s="0"/>
-      <c r="K69" s="0"/>
-      <c r="L69" s="0"/>
-      <c r="M69" s="0"/>
-      <c r="N69" s="1"/>
-      <c r="O69" s="1"/>
-      <c r="P69" s="1"/>
-      <c r="Q69" s="1"/>
-      <c r="R69" s="1"/>
-      <c r="X69" s="1"/>
-      <c r="Y69" s="1"/>
-      <c r="Z69" s="1"/>
-      <c r="AA69" s="1"/>
-      <c r="AB69" s="1"/>
+      <c r="A69" s="3"/>
+      <c r="B69" s="3"/>
+      <c r="D69" s="3"/>
+      <c r="E69" s="3"/>
+      <c r="F69" s="3"/>
+      <c r="G69" s="3"/>
+      <c r="H69" s="3"/>
+      <c r="I69" s="3"/>
+      <c r="J69" s="3"/>
+      <c r="K69" s="3"/>
+      <c r="L69" s="3"/>
+      <c r="M69" s="3"/>
     </row>
     <row r="70" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A70" s="0"/>
-      <c r="B70" s="0"/>
-      <c r="D70" s="0"/>
-      <c r="E70" s="0"/>
-      <c r="F70" s="0"/>
-      <c r="G70" s="0"/>
-      <c r="H70" s="0"/>
-      <c r="I70" s="0"/>
-      <c r="J70" s="0"/>
-      <c r="K70" s="0"/>
-      <c r="L70" s="0"/>
-      <c r="M70" s="0"/>
-      <c r="N70" s="1"/>
-      <c r="O70" s="1"/>
-      <c r="P70" s="1"/>
-      <c r="Q70" s="1"/>
-      <c r="R70" s="1"/>
-      <c r="X70" s="1"/>
-      <c r="Y70" s="1"/>
-      <c r="Z70" s="1"/>
-      <c r="AA70" s="1"/>
-      <c r="AB70" s="1"/>
+      <c r="A70" s="3"/>
+      <c r="B70" s="3"/>
+      <c r="D70" s="3"/>
+      <c r="E70" s="3"/>
+      <c r="F70" s="3"/>
+      <c r="G70" s="3"/>
+      <c r="H70" s="3"/>
+      <c r="I70" s="3"/>
+      <c r="J70" s="3"/>
+      <c r="K70" s="3"/>
+      <c r="L70" s="3"/>
+      <c r="M70" s="3"/>
     </row>
     <row r="71" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A71" s="0"/>
-      <c r="B71" s="0"/>
-      <c r="D71" s="0"/>
-      <c r="E71" s="0"/>
-      <c r="F71" s="0"/>
-      <c r="G71" s="0"/>
-      <c r="H71" s="0"/>
-      <c r="I71" s="0"/>
-      <c r="J71" s="0"/>
-      <c r="K71" s="0"/>
-      <c r="L71" s="0"/>
-      <c r="M71" s="0"/>
-      <c r="N71" s="1"/>
-      <c r="O71" s="1"/>
-      <c r="P71" s="1"/>
-      <c r="Q71" s="1"/>
-      <c r="R71" s="1"/>
-      <c r="X71" s="1"/>
-      <c r="Y71" s="1"/>
-      <c r="Z71" s="1"/>
-      <c r="AA71" s="1"/>
-      <c r="AB71" s="1"/>
+      <c r="A71" s="3"/>
+      <c r="B71" s="3"/>
+      <c r="D71" s="3"/>
+      <c r="E71" s="3"/>
+      <c r="F71" s="3"/>
+      <c r="G71" s="3"/>
+      <c r="H71" s="3"/>
+      <c r="I71" s="3"/>
+      <c r="J71" s="3"/>
+      <c r="K71" s="3"/>
+      <c r="L71" s="3"/>
+      <c r="M71" s="3"/>
     </row>
     <row r="72" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A72" s="0"/>
-      <c r="B72" s="0"/>
-      <c r="D72" s="0"/>
-      <c r="E72" s="0"/>
-      <c r="F72" s="0"/>
-      <c r="G72" s="0"/>
-      <c r="H72" s="0"/>
-      <c r="I72" s="0"/>
-      <c r="J72" s="0"/>
-      <c r="K72" s="0"/>
-      <c r="L72" s="0"/>
-      <c r="M72" s="0"/>
-      <c r="AA72" s="1"/>
+      <c r="A72" s="3"/>
+      <c r="B72" s="3"/>
+      <c r="D72" s="3"/>
+      <c r="E72" s="3"/>
+      <c r="F72" s="3"/>
+      <c r="G72" s="3"/>
+      <c r="H72" s="3"/>
+      <c r="I72" s="3"/>
+      <c r="J72" s="3"/>
+      <c r="K72" s="3"/>
+      <c r="L72" s="3"/>
+      <c r="M72" s="3"/>
     </row>
     <row r="73" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A73" s="0"/>
-      <c r="B73" s="0"/>
-      <c r="D73" s="0"/>
-      <c r="E73" s="0"/>
-      <c r="F73" s="0"/>
-      <c r="G73" s="0"/>
-      <c r="H73" s="0"/>
-      <c r="I73" s="0"/>
-      <c r="J73" s="0"/>
-      <c r="K73" s="0"/>
-      <c r="L73" s="0"/>
-      <c r="M73" s="0"/>
+      <c r="A73" s="3"/>
+      <c r="B73" s="3"/>
+      <c r="D73" s="3"/>
+      <c r="E73" s="3"/>
+      <c r="F73" s="3"/>
+      <c r="G73" s="3"/>
+      <c r="H73" s="3"/>
+      <c r="I73" s="3"/>
+      <c r="J73" s="3"/>
+      <c r="K73" s="3"/>
+      <c r="L73" s="3"/>
+      <c r="M73" s="3"/>
     </row>
     <row r="74" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A74" s="0"/>
-      <c r="B74" s="0"/>
-      <c r="D74" s="0"/>
-      <c r="E74" s="0"/>
-      <c r="F74" s="0"/>
-      <c r="G74" s="0"/>
-      <c r="H74" s="0"/>
-      <c r="I74" s="0"/>
-      <c r="J74" s="0"/>
-      <c r="K74" s="0"/>
-      <c r="L74" s="0"/>
-      <c r="M74" s="0"/>
+      <c r="A74" s="3"/>
+      <c r="B74" s="3"/>
+      <c r="D74" s="3"/>
+      <c r="E74" s="3"/>
+      <c r="F74" s="3"/>
+      <c r="G74" s="3"/>
+      <c r="H74" s="3"/>
+      <c r="I74" s="3"/>
+      <c r="J74" s="3"/>
+      <c r="K74" s="3"/>
+      <c r="L74" s="3"/>
+      <c r="M74" s="3"/>
     </row>
     <row r="75" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A75" s="0"/>
-      <c r="B75" s="0"/>
-      <c r="D75" s="0"/>
-      <c r="E75" s="0"/>
-      <c r="F75" s="0"/>
-      <c r="G75" s="0"/>
-      <c r="H75" s="0"/>
-      <c r="I75" s="0"/>
-      <c r="J75" s="0"/>
-      <c r="K75" s="0"/>
-      <c r="L75" s="0"/>
-      <c r="M75" s="0"/>
+      <c r="A75" s="3"/>
+      <c r="B75" s="3"/>
+      <c r="D75" s="3"/>
+      <c r="E75" s="3"/>
+      <c r="F75" s="3"/>
+      <c r="G75" s="3"/>
+      <c r="H75" s="3"/>
+      <c r="I75" s="3"/>
+      <c r="J75" s="3"/>
+      <c r="K75" s="3"/>
+      <c r="L75" s="3"/>
+      <c r="M75" s="3"/>
     </row>
     <row r="76" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A76" s="0"/>
-      <c r="B76" s="0"/>
-      <c r="D76" s="0"/>
-      <c r="E76" s="0"/>
-      <c r="F76" s="0"/>
-      <c r="G76" s="0"/>
-      <c r="H76" s="0"/>
-      <c r="I76" s="0"/>
-      <c r="J76" s="0"/>
-      <c r="K76" s="0"/>
-      <c r="L76" s="0"/>
-      <c r="M76" s="0"/>
+      <c r="A76" s="3"/>
+      <c r="B76" s="3"/>
+      <c r="D76" s="3"/>
+      <c r="E76" s="3"/>
+      <c r="F76" s="3"/>
+      <c r="G76" s="3"/>
+      <c r="H76" s="3"/>
+      <c r="I76" s="3"/>
+      <c r="J76" s="3"/>
+      <c r="K76" s="3"/>
+      <c r="L76" s="3"/>
+      <c r="M76" s="3"/>
     </row>
     <row r="77" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A77" s="0"/>
-      <c r="B77" s="0"/>
-      <c r="D77" s="0"/>
-      <c r="E77" s="0"/>
-      <c r="F77" s="0"/>
-      <c r="G77" s="0"/>
-      <c r="H77" s="0"/>
-      <c r="I77" s="0"/>
-      <c r="J77" s="0"/>
-      <c r="K77" s="0"/>
-      <c r="L77" s="0"/>
-      <c r="M77" s="0"/>
+      <c r="A77" s="3"/>
+      <c r="B77" s="3"/>
+      <c r="D77" s="3"/>
+      <c r="E77" s="3"/>
+      <c r="F77" s="3"/>
+      <c r="G77" s="3"/>
+      <c r="H77" s="3"/>
+      <c r="I77" s="3"/>
+      <c r="J77" s="3"/>
+      <c r="K77" s="3"/>
+      <c r="L77" s="3"/>
+      <c r="M77" s="3"/>
     </row>
     <row r="78" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A78" s="0"/>
-      <c r="B78" s="0"/>
-      <c r="D78" s="0"/>
-      <c r="E78" s="0"/>
-      <c r="F78" s="0"/>
-      <c r="G78" s="0"/>
-      <c r="H78" s="0"/>
-      <c r="I78" s="0"/>
-      <c r="J78" s="0"/>
-      <c r="K78" s="0"/>
-      <c r="L78" s="0"/>
-      <c r="M78" s="0"/>
+      <c r="A78" s="3"/>
+      <c r="B78" s="3"/>
+      <c r="D78" s="3"/>
+      <c r="E78" s="3"/>
+      <c r="F78" s="3"/>
+      <c r="G78" s="3"/>
+      <c r="H78" s="3"/>
+      <c r="I78" s="3"/>
+      <c r="J78" s="3"/>
+      <c r="K78" s="3"/>
+      <c r="L78" s="3"/>
+      <c r="M78" s="3"/>
     </row>
     <row r="79" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A79" s="0"/>
-      <c r="B79" s="0"/>
-      <c r="D79" s="0"/>
-      <c r="E79" s="0"/>
-      <c r="F79" s="0"/>
-      <c r="G79" s="0"/>
-      <c r="H79" s="0"/>
-      <c r="I79" s="0"/>
-      <c r="J79" s="0"/>
-      <c r="K79" s="0"/>
-      <c r="L79" s="0"/>
-      <c r="M79" s="0"/>
+      <c r="A79" s="3"/>
+      <c r="B79" s="3"/>
+      <c r="D79" s="3"/>
+      <c r="E79" s="3"/>
+      <c r="F79" s="3"/>
+      <c r="G79" s="3"/>
+      <c r="H79" s="3"/>
+      <c r="I79" s="3"/>
+      <c r="J79" s="3"/>
+      <c r="K79" s="3"/>
+      <c r="L79" s="3"/>
+      <c r="M79" s="3"/>
     </row>
     <row r="80" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A80" s="0"/>
-      <c r="B80" s="0"/>
-      <c r="D80" s="0"/>
-      <c r="E80" s="0"/>
-      <c r="F80" s="0"/>
-      <c r="G80" s="0"/>
-      <c r="H80" s="0"/>
-      <c r="I80" s="0"/>
-      <c r="J80" s="0"/>
-      <c r="K80" s="0"/>
-      <c r="L80" s="0"/>
-      <c r="M80" s="0"/>
+      <c r="A80" s="3"/>
+      <c r="B80" s="3"/>
+      <c r="D80" s="3"/>
+      <c r="E80" s="3"/>
+      <c r="F80" s="3"/>
+      <c r="G80" s="3"/>
+      <c r="H80" s="3"/>
+      <c r="I80" s="3"/>
+      <c r="J80" s="3"/>
+      <c r="K80" s="3"/>
+      <c r="L80" s="3"/>
+      <c r="M80" s="3"/>
     </row>
     <row r="81" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A81" s="0"/>
-      <c r="B81" s="0"/>
-      <c r="D81" s="0"/>
-      <c r="E81" s="0"/>
-      <c r="F81" s="0"/>
-      <c r="G81" s="0"/>
-      <c r="H81" s="0"/>
-      <c r="I81" s="0"/>
-      <c r="J81" s="0"/>
-      <c r="K81" s="0"/>
-      <c r="L81" s="0"/>
-      <c r="M81" s="0"/>
+      <c r="A81" s="3"/>
+      <c r="B81" s="3"/>
+      <c r="D81" s="3"/>
+      <c r="E81" s="3"/>
+      <c r="F81" s="3"/>
+      <c r="G81" s="3"/>
+      <c r="H81" s="3"/>
+      <c r="I81" s="3"/>
+      <c r="J81" s="3"/>
+      <c r="K81" s="3"/>
+      <c r="L81" s="3"/>
+      <c r="M81" s="3"/>
     </row>
     <row r="82" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A82" s="0"/>
-      <c r="B82" s="0"/>
-      <c r="D82" s="0"/>
-      <c r="E82" s="0"/>
-      <c r="F82" s="0"/>
-      <c r="G82" s="0"/>
-      <c r="H82" s="0"/>
-      <c r="I82" s="0"/>
-      <c r="J82" s="0"/>
-      <c r="K82" s="0"/>
-      <c r="L82" s="0"/>
-      <c r="M82" s="0"/>
+      <c r="A82" s="3"/>
+      <c r="B82" s="3"/>
+      <c r="D82" s="3"/>
+      <c r="E82" s="3"/>
+      <c r="F82" s="3"/>
+      <c r="G82" s="3"/>
+      <c r="H82" s="3"/>
+      <c r="I82" s="3"/>
+      <c r="J82" s="3"/>
+      <c r="K82" s="3"/>
+      <c r="L82" s="3"/>
+      <c r="M82" s="3"/>
     </row>
     <row r="83" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A83" s="0"/>
-      <c r="B83" s="0"/>
-      <c r="D83" s="0"/>
-      <c r="E83" s="0"/>
-      <c r="F83" s="0"/>
-      <c r="G83" s="0"/>
-      <c r="H83" s="0"/>
-      <c r="I83" s="0"/>
-      <c r="J83" s="0"/>
-      <c r="K83" s="0"/>
-      <c r="L83" s="0"/>
-      <c r="M83" s="0"/>
+      <c r="A83" s="3"/>
+      <c r="B83" s="3"/>
+      <c r="D83" s="3"/>
+      <c r="E83" s="3"/>
+      <c r="F83" s="3"/>
+      <c r="G83" s="3"/>
+      <c r="H83" s="3"/>
+      <c r="I83" s="3"/>
+      <c r="J83" s="3"/>
+      <c r="K83" s="3"/>
+      <c r="L83" s="3"/>
+      <c r="M83" s="3"/>
     </row>
     <row r="84" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A84" s="0"/>
-      <c r="B84" s="0"/>
-      <c r="D84" s="0"/>
-      <c r="E84" s="0"/>
-      <c r="F84" s="0"/>
-      <c r="G84" s="0"/>
-      <c r="H84" s="0"/>
-      <c r="I84" s="0"/>
-      <c r="J84" s="0"/>
-      <c r="K84" s="0"/>
-      <c r="L84" s="0"/>
-      <c r="M84" s="0"/>
+      <c r="A84" s="3"/>
+      <c r="B84" s="3"/>
+      <c r="D84" s="3"/>
+      <c r="E84" s="3"/>
+      <c r="F84" s="3"/>
+      <c r="G84" s="3"/>
+      <c r="H84" s="3"/>
+      <c r="I84" s="3"/>
+      <c r="J84" s="3"/>
+      <c r="K84" s="3"/>
+      <c r="L84" s="3"/>
+      <c r="M84" s="3"/>
     </row>
     <row r="85" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A85" s="0"/>
-      <c r="B85" s="0"/>
-      <c r="D85" s="0"/>
-      <c r="E85" s="0"/>
-      <c r="F85" s="0"/>
-      <c r="G85" s="0"/>
-      <c r="H85" s="0"/>
-      <c r="I85" s="0"/>
-      <c r="J85" s="0"/>
-      <c r="K85" s="0"/>
-      <c r="L85" s="0"/>
-      <c r="M85" s="0"/>
+      <c r="A85" s="3"/>
+      <c r="B85" s="3"/>
+      <c r="D85" s="3"/>
+      <c r="E85" s="3"/>
+      <c r="F85" s="3"/>
+      <c r="G85" s="3"/>
+      <c r="H85" s="3"/>
+      <c r="I85" s="3"/>
+      <c r="J85" s="3"/>
+      <c r="K85" s="3"/>
+      <c r="L85" s="3"/>
+      <c r="M85" s="3"/>
     </row>
     <row r="86" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A86" s="0"/>
-      <c r="B86" s="0"/>
-      <c r="D86" s="0"/>
-      <c r="E86" s="0"/>
-      <c r="F86" s="0"/>
-      <c r="G86" s="0"/>
-      <c r="H86" s="0"/>
-      <c r="I86" s="0"/>
-      <c r="J86" s="0"/>
-      <c r="K86" s="0"/>
-      <c r="L86" s="0"/>
-      <c r="M86" s="0"/>
+      <c r="A86" s="3"/>
+      <c r="B86" s="3"/>
+      <c r="D86" s="3"/>
+      <c r="E86" s="3"/>
+      <c r="F86" s="3"/>
+      <c r="G86" s="3"/>
+      <c r="H86" s="3"/>
+      <c r="I86" s="3"/>
+      <c r="J86" s="3"/>
+      <c r="K86" s="3"/>
+      <c r="L86" s="3"/>
+      <c r="M86" s="3"/>
     </row>
     <row r="87" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A87" s="0"/>
-      <c r="B87" s="0"/>
-      <c r="D87" s="0"/>
-      <c r="E87" s="0"/>
-      <c r="F87" s="0"/>
-      <c r="G87" s="0"/>
-      <c r="H87" s="0"/>
-      <c r="I87" s="0"/>
-      <c r="J87" s="0"/>
-      <c r="K87" s="0"/>
-      <c r="L87" s="0"/>
-      <c r="M87" s="0"/>
+      <c r="A87" s="3"/>
+      <c r="B87" s="3"/>
+      <c r="D87" s="3"/>
+      <c r="E87" s="3"/>
+      <c r="F87" s="3"/>
+      <c r="G87" s="3"/>
+      <c r="H87" s="3"/>
+      <c r="I87" s="3"/>
+      <c r="J87" s="3"/>
+      <c r="K87" s="3"/>
+      <c r="L87" s="3"/>
+      <c r="M87" s="3"/>
     </row>
     <row r="88" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A88" s="0"/>
-      <c r="B88" s="0"/>
-      <c r="D88" s="0"/>
-      <c r="E88" s="0"/>
-      <c r="F88" s="0"/>
-      <c r="G88" s="0"/>
-      <c r="H88" s="0"/>
-      <c r="I88" s="0"/>
-      <c r="J88" s="0"/>
-      <c r="K88" s="0"/>
-      <c r="L88" s="0"/>
-      <c r="M88" s="0"/>
+      <c r="A88" s="3"/>
+      <c r="B88" s="3"/>
+      <c r="D88" s="3"/>
+      <c r="E88" s="3"/>
+      <c r="F88" s="3"/>
+      <c r="G88" s="3"/>
+      <c r="H88" s="3"/>
+      <c r="I88" s="3"/>
+      <c r="J88" s="3"/>
+      <c r="K88" s="3"/>
+      <c r="L88" s="3"/>
+      <c r="M88" s="3"/>
     </row>
     <row r="89" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A89" s="0"/>
-      <c r="B89" s="0"/>
-      <c r="D89" s="0"/>
-      <c r="E89" s="0"/>
-      <c r="F89" s="0"/>
-      <c r="G89" s="0"/>
-      <c r="H89" s="0"/>
-      <c r="I89" s="0"/>
-      <c r="J89" s="0"/>
-      <c r="K89" s="0"/>
-      <c r="L89" s="0"/>
-      <c r="M89" s="0"/>
+      <c r="A89" s="3"/>
+      <c r="B89" s="3"/>
+      <c r="D89" s="3"/>
+      <c r="E89" s="3"/>
+      <c r="F89" s="3"/>
+      <c r="G89" s="3"/>
+      <c r="H89" s="3"/>
+      <c r="I89" s="3"/>
+      <c r="J89" s="3"/>
+      <c r="K89" s="3"/>
+      <c r="L89" s="3"/>
+      <c r="M89" s="3"/>
     </row>
     <row r="90" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A90" s="0"/>
-      <c r="B90" s="0"/>
-      <c r="D90" s="0"/>
-      <c r="E90" s="0"/>
-      <c r="F90" s="0"/>
-      <c r="G90" s="0"/>
-      <c r="H90" s="0"/>
-      <c r="I90" s="0"/>
-      <c r="J90" s="0"/>
-      <c r="K90" s="0"/>
-      <c r="L90" s="0"/>
-      <c r="M90" s="0"/>
+      <c r="A90" s="3"/>
+      <c r="B90" s="3"/>
+      <c r="D90" s="3"/>
+      <c r="E90" s="3"/>
+      <c r="F90" s="3"/>
+      <c r="G90" s="3"/>
+      <c r="H90" s="3"/>
+      <c r="I90" s="3"/>
+      <c r="J90" s="3"/>
+      <c r="K90" s="3"/>
+      <c r="L90" s="3"/>
+      <c r="M90" s="3"/>
     </row>
     <row r="91" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A91" s="0"/>
-      <c r="B91" s="0"/>
-      <c r="D91" s="0"/>
-      <c r="E91" s="0"/>
-      <c r="F91" s="0"/>
-      <c r="G91" s="0"/>
-      <c r="H91" s="0"/>
-      <c r="I91" s="0"/>
-      <c r="J91" s="0"/>
-      <c r="K91" s="0"/>
-      <c r="L91" s="0"/>
-      <c r="M91" s="0"/>
+      <c r="A91" s="3"/>
+      <c r="B91" s="3"/>
+      <c r="D91" s="3"/>
+      <c r="E91" s="3"/>
+      <c r="F91" s="3"/>
+      <c r="G91" s="3"/>
+      <c r="H91" s="3"/>
+      <c r="I91" s="3"/>
+      <c r="J91" s="3"/>
+      <c r="K91" s="3"/>
+      <c r="L91" s="3"/>
+      <c r="M91" s="3"/>
     </row>
     <row r="92" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A92" s="0"/>
-      <c r="B92" s="0"/>
-      <c r="D92" s="0"/>
-      <c r="E92" s="0"/>
-      <c r="F92" s="0"/>
-      <c r="G92" s="0"/>
-      <c r="H92" s="0"/>
-      <c r="I92" s="0"/>
-      <c r="J92" s="0"/>
-      <c r="K92" s="0"/>
-      <c r="L92" s="0"/>
-      <c r="M92" s="0"/>
+      <c r="A92" s="3"/>
+      <c r="B92" s="3"/>
+      <c r="D92" s="3"/>
+      <c r="E92" s="3"/>
+      <c r="F92" s="3"/>
+      <c r="G92" s="3"/>
+      <c r="H92" s="3"/>
+      <c r="I92" s="3"/>
+      <c r="J92" s="3"/>
+      <c r="K92" s="3"/>
+      <c r="L92" s="3"/>
+      <c r="M92" s="3"/>
     </row>
     <row r="93" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A93" s="0"/>
-      <c r="B93" s="0"/>
-      <c r="D93" s="0"/>
-      <c r="E93" s="0"/>
-      <c r="F93" s="0"/>
-      <c r="G93" s="0"/>
-      <c r="H93" s="0"/>
-      <c r="K93" s="1"/>
-      <c r="L93" s="1"/>
+      <c r="A93" s="3"/>
+      <c r="B93" s="3"/>
+      <c r="D93" s="3"/>
+      <c r="E93" s="3"/>
+      <c r="F93" s="3"/>
+      <c r="G93" s="3"/>
+      <c r="H93" s="3"/>
     </row>
     <row r="94" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A94" s="0"/>
-      <c r="B94" s="0"/>
-      <c r="D94" s="0"/>
-      <c r="E94" s="0"/>
-      <c r="F94" s="0"/>
-      <c r="G94" s="0"/>
-      <c r="H94" s="0"/>
-      <c r="K94" s="1"/>
-      <c r="L94" s="1"/>
+      <c r="A94" s="3"/>
+      <c r="B94" s="3"/>
+      <c r="D94" s="3"/>
+      <c r="E94" s="3"/>
+      <c r="F94" s="3"/>
+      <c r="G94" s="3"/>
+      <c r="H94" s="3"/>
     </row>
     <row r="95" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="E95" s="0"/>
-      <c r="K95" s="1"/>
-      <c r="L95" s="1"/>
+      <c r="E95" s="3"/>
     </row>
     <row r="96" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="E96" s="0"/>
-      <c r="K96" s="1"/>
-      <c r="L96" s="1"/>
+      <c r="E96" s="3"/>
     </row>
     <row r="97" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="E97" s="0"/>
-      <c r="K97" s="1"/>
-      <c r="L97" s="1"/>
+      <c r="E97" s="3"/>
     </row>
     <row r="98" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="E98" s="0"/>
-      <c r="K98" s="1"/>
+      <c r="E98" s="3"/>
     </row>
     <row r="99" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="E99" s="0"/>
-      <c r="K99" s="1"/>
+      <c r="E99" s="3"/>
     </row>
     <row r="100" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="E100" s="0"/>
-      <c r="K100" s="1"/>
+      <c r="E100" s="3"/>
     </row>
     <row r="101" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="E101" s="0"/>
-      <c r="I101" s="1"/>
-      <c r="K101" s="1"/>
+      <c r="E101" s="3"/>
     </row>
     <row r="102" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="E102" s="0"/>
-      <c r="I102" s="1"/>
-      <c r="K102" s="1"/>
+      <c r="E102" s="3"/>
     </row>
     <row r="103" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="E103" s="0"/>
-      <c r="I103" s="1"/>
-      <c r="K103" s="1"/>
+      <c r="E103" s="3"/>
     </row>
     <row r="104" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="E104" s="0"/>
-      <c r="I104" s="1"/>
-      <c r="K104" s="1"/>
+      <c r="E104" s="3"/>
     </row>
     <row r="105" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="E105" s="0"/>
-      <c r="I105" s="1"/>
-      <c r="J105" s="1"/>
-      <c r="K105" s="1"/>
+      <c r="E105" s="3"/>
     </row>
     <row r="106" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="E106" s="0"/>
+      <c r="E106" s="3"/>
     </row>
     <row r="107" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="E107" s="0"/>
+      <c r="E107" s="3"/>
     </row>
     <row r="108" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="E108" s="0"/>
+      <c r="E108" s="3"/>
     </row>
     <row r="109" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="E109" s="0"/>
+      <c r="E109" s="3"/>
     </row>
     <row r="110" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="E110" s="0"/>
+      <c r="E110" s="3"/>
     </row>
     <row r="111" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="E111" s="0"/>
+      <c r="E111" s="3"/>
     </row>
     <row r="112" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="E112" s="0"/>
+      <c r="E112" s="3"/>
     </row>
     <row r="113" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="E113" s="0"/>
+      <c r="E113" s="3"/>
     </row>
     <row r="114" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="E114" s="0"/>
-      <c r="H114" s="1"/>
+      <c r="E114" s="3"/>
     </row>
     <row r="115" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="E115" s="0"/>
-      <c r="H115" s="1"/>
+      <c r="E115" s="3"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
add answers given in the downloadable report
</commit_message>
<xml_diff>
--- a/report_template_simplified.xlsx
+++ b/report_template_simplified.xlsx
@@ -8,8 +8,8 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Foglio1" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Foglio2" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Risultati" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Risposte" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="97">
   <si>
     <t xml:space="preserve">Punteggio complessivo</t>
   </si>
@@ -87,6 +87,231 @@
   </si>
   <si>
     <t xml:space="preserve">Sì</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Domanda:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Risposta:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Descrizione:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto-valutazione:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Priorità:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Note:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione implementa pratiche di incentivazione strettamente connessi ai cambiamenti climantici nella remunerazione dei membri degli organi di Amministrazione, Direzione e Controllo?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E' presente un piano di transizione per la mitigazione dei cambiamenti climatici? Nello specifico, l'Azienda allinea la strategia e il modello aziendale alla limitazione del riscaldamento globale a 1,5 °C conformemente alle disposizioni disciplinate dall'accordo di Parigi?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione identifica e valuta gli impatti, i rischi e le opportunità legati ai cambiamenti climatici? Se si, come vengono gestiti?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sono presenti delle politiche ed azioni specifiche intraprese per mitigare e adattarsi ai cambiamenti climatici? Quali risorse sono state allocate per queste politiche e azioni?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione ha stabilito obiettivi specifici per la mitigazione dei cambiamenti climatici e l'adattamento agli stessi?​​</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione monitora il consumo di energia tenendo conto del relativo mix energetico?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vengono misurate le emissioni lorde di gas serra (GHG) di Scope 1, 2, e 3 e le emissioni totali di GHG? Esistono progetti di mitigazione delle stesse?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione ha identificato gli effetti finanziari derivati dai rischi e dalle opportunità legati al cambiamento climatico? (ad esempio tenendo conto della influenza sulla situazione patrimoniale-finanziaria, sul risultato economico e sui flussi finanziari dell'impresa nel breve, medio e lungo periodo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione identifica e valuta gli impatti, i rischi e le opportunità legati all'inquinamento di aria, acqua e suolo? Se si, come vengono gestiti?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione ha adottato delle politiche per la gestione dell'inquinamento? Se si, quali risorse sono state allocate a sostegno di queste politiche? Quali azioni sono state intraprese per prevenire, ridurre o controllare l'inquinamento?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sono stati fissati degli obiettivi specifici per prevenire, ridurre o controllare l'inquinamento e monitorare il loro progresso?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vengono misurate e riportate le emissioni di inquinanti nell'aria, nell'acqua e nel suolo?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vengono pubblicate informazioni inerenti le quantità delle sostanze preoccupanti ed estremamente preoccupanti prodotte, utilizzate o commercializzate dall'Organizzazione?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione ha identificato gli effetti finanziari attesi derivati da rischi e opportunità legati all'inquinamento?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione identifica e valuta gli impatti, i rischi e le opportunità legati alle acque e alle risorse marine? Se si, come vengono gestiti?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione ha adottato delle politiche per la gestione delle acque e delle risorse marine? Se si, quali risorse sono state allocate a sostegno di queste politiche? Quali azioni sono state intraprese per prevenire, ridurre o controllare gli impatti sulle acque e sulle risorse marine?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sono stati fissati degli obiettivi specifici per gestire gli impatti sulle acque e sulle risorse marine e monitorare il progresso verso questi obiettivi?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vengono misurati e riportati il consumo di acqua e gli scarichi idrici dell'azienda?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione ha identificato gli effetti finanziari attesi derivanti da rischi e opportunità legati alle acque e alle risorse marine?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione descrive la resilienza della propria strategia e del proprio modello aziendale in relazione alla biodiversità e agli ecosistemi?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'organizzazione ha individuato le attività che incidono negativamente sulle aree sensibili sotto il profilo della biodiversità?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione identifica e valuta gli impatti, i rischi e le opportunità legati alla biodiversità e agli ecosistemi?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione ha adottato delle politiche per la gestione degli impatti, rischi e dipendenze in termini di biodiversità ed ecosistemi? Se si, quali risorse sono state allocate a sostegno di queste politiche? Quali azioni sono state intraprese per prevenire, ridurre o controllare gli impatti sulla biodiversità e sugli ecosistemi?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione ha fissato obiettivi connessi alla biodiversità e agli ecosistemi? Viene monitorato il progresso verso il loro raggiungimento?​​</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione ha identificato delle metriche per monitorare gli impatti legati ai cambiamenti della biodiversità e degli ecosistemi?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione ha identificato gli effetti finanziari attesi derivanti da rischi e opportunità connessi alla biodiversità e agli ecosistemi?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione identifica e valuta gli impatti, i rischi e le opportunità legati all'uso delle risorse e all'economia circolare? Se si, come vengono gestiti?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione ha adottato delle politiche per la gestione delle risorse e dell'economia circolare? Se si, quali risorse sono state allocate a sostegno di queste politiche? Quali azioni sono state intraprese  per promuovere l'uso efficiente delle risorse e delle pratiche di economia circolare?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sono stati fissati degli obiettivi specifici connessi all'uso delle risorse e all'economia circolare? Viene monitorato progresso di tali obiettivi?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vengono misurati e riportati i flussi di risorse in entrata e in uscita, compresi i prodotti, i materiali e i rifiuti? Queste voci vengono messe in relazione ai propri impatti, rischi e opportunità rilevanti?​</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione ha identificato gli effetti finanziari attesi derivati da rischi e opportunità connessi all'uso delle risorse e all'economia circolare?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vengono integrate questioni relative alla forza lavoro propria nella strategia e nel modello di business aziendale? (Condizioni di lavoro sicure, salari adeguati e parità di trattamento con relativa prevenzione alla discriminazione…)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione ha adottato politiche per gestire i suoi impatti significativi sulla forza lavoro, inclusi i rischi e le opportunità?​​ Se si, come sono coinvolti i lavoratori e i loro rappresentanti nel processo decisionale riguardante tali impatti?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sono stati definiti dei processi per porre rimedio agli impatti negativi sui lavoratori? Sono disponibili canali specifici che i lavoratori possono utilizzare per sollevare le loro preoccupazioni e far si che queste vengano trattate?​</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione ha fissato obiettivi per gestire gli impatti negativi, potenziare gli impatti positivi, e gestire i rischi e le opportunità legati alla forza lavoro propria?​​</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione descrive le caratteristiche dei propri dipendenti, inclusi i dettagli su contratti? (a tempo indeterminato, a tempo parziale, tassi di avvicendamento dei dipendenti...)​</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione rende nota la percentuale dei dipendenti coperta da contratti collettivi e non? Viene promosso il dialogo sociale all'interno dell'Organizzazione?​​</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quali delle seguenti metriche sono monitorate dall'Organizzazione:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distribuzione di genere tra i membri dell'alta dirigenza</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distribuzione per età dei suoi dipendenti</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Numero di dipendenti coperti dalla protezione sociale (malattia, disoccupazione, infortuni, congedi, pensionamenti…)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Percentuale di dipendenti con disabilità</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Percentuale di dipendenti che hanno usufruito di ore di formazione e sviluppo delle competenze</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Percentuale delle sedi in capo all'Organizzazione coperte da un sistema di gestione della salute e sicurezza sui luoghi di lavoro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Percentuale dei dipendenti che hanno diritto a congedo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Divario tra remunerazioni per sesso maschile e femminile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Numero di incidenti, denunce e impatti gravi in materia di diritti umani</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vengono integrate nella strategia e nel modello di business aziendale questioni relative ai lavoratori nella catena del valore? (Condizioni di lavoro sicure, salari adeguati e parità di trattamento con relativa prevenzione alla discriminazione…)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione ha adottato politiche per gestire i suoi impatti significativi sui lavoratori nella catena del valore, inclusi i rischi e le opportunità associati?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vengono coinvolti dall'Organizzazione i lavoratori nella catena del valore e i loro rappresentanti in merito agli impatti, effettivi e potenziali, che li riguardano?​​</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione interviene per far fronte agli impatti, gestire i rischi e le opportunità rilevanti per i lavoratori nella catena del valore? Viene monitorata l'efficacia di tali azioni?​​</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione ha fissato obiettivi per gestire gli impatti negativi, potenziare gli impatti positivi, e gestire i rischi e le opportunità legati ai lavoratori nella catena del valore?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione orienta la sua strategia tenendo conto delle motivazioni che coinvolgono le comunità interessate? (Locali e distanti)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione ha adottato politiche per gestire i suoi impatti significativi sulle comunità interessate, inclusi i rischi e le opportunità associati?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione ha coinvolto le comunità interessate e i loro rappresentanti, in merito agli impatti rilevanti, sia positivi che negativi, che le riguardano o potrebbero riguardarle?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione interviene per far fronte agli impatti, gestire i rischi e le opportunità rilevanti per le comunità interessate? Viene monitorata l'efficacia di tali azioni?​​</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione ha fissato obiettivi per gestire gli impatti negativi, potenziare gli impatti positivi, e gestire i rischi e le opportunità sulle comunità interessate?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vengono integrate nella strategia e nel modello di business aziendale questioni relative ai  consumatori e/o agli utilizzatori finali? (Es: danni al consumatore dovuti al prodotto/servizio offerto, se il prodotto/servizio necessita di specifici manuali o etichette…)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione ha adottato politiche per gestire gli impatti dei suoi prodotti e/o servizi sui consumatori e sugli utilizzatori finali, compresi i rischi e le opportunità rilevanti associati? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione ha predisposto processi volti a coinvolgere i consumatori e/o gli utilizzatori finali in merito agli impatti rilevanti che li riguardano, sia positivi che negativi? Se si, ha messo in atto dei processi per porre rimedio ad eventuali impatti negativi?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione interviene per far fronte agli impatti, gestire i rischi e le opportunità rilevanti sui consumatori e sugli utilizzatori finali? Viene monitorata l'efficacia di tali azioni?​​</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sono stati implementati degli obiettivi temporali e orientati ai risultati per la riduzione degli impatti negativi sui consumatori e/o sugli utilizzatori finali e/o per il potenziamento degli impatti positivi sui consumatori e/o sugli utilizzatori finali?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione descrive il ruolo degli organi di Amministrazione-Direzione-Controllo in relazione alle tematiche della condotta d'impresa? ( Etica aziendale, corruzione, cultura d'impresa, rapporti con i fornitori comprese prassi di pagamento, influenza politica, attività di lobbying...)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione ha adottato politiche per promuovere una cultura d'impresa etica e responsabile? (codici di condotta, sistemi di gestione accreditati per contrastare la corruzione…)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione individua, valuta, gestisce e/o porge rimedio ai propri impatti, rischi e opportunità connessi alle questioni di condotta delle imprese?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sono stati implementati processi per gestire i rapporti con i fornitori in modo etico e sostenibile?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione ha adottato misure per prevenire e individuare prassi di corruzione, sia attiva che passiva?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione quantifica i casi di corruzione, sia attiva che passiva?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Organizzazione si impegna in modo trasparente e responsabile nelle attività di lobbying e di influenza politica? Vengono quantificati i valori monetari dei contributi forniti direttamente dall'impresa?</t>
   </si>
 </sst>
 </file>
@@ -96,7 +321,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="9">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -130,8 +355,29 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b val="true"/>
+      <i val="true"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="20"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -153,7 +399,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFD7"/>
-        <bgColor rgb="FFEEEEEE"/>
+        <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -168,13 +414,26 @@
         <bgColor rgb="FFEEEEEE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor rgb="FFFFFFD7"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
   </borders>
@@ -203,7 +462,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="17">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -236,6 +495,42 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -248,7 +543,7 @@
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
-      <rgbColor rgb="FFEEEEEE"/>
+      <rgbColor rgb="FFFFFFFF"/>
       <rgbColor rgb="FFFF0000"/>
       <rgbColor rgb="FF00FF00"/>
       <rgbColor rgb="FF0000FF"/>
@@ -280,7 +575,7 @@
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FF80FF80"/>
+      <rgbColor rgb="FFEEEEEE"/>
       <rgbColor rgb="FFDDE8CB"/>
       <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FFA0E0A0"/>
@@ -289,7 +584,7 @@
       <rgbColor rgb="FFFFC080"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
-      <rgbColor rgb="FF99CC00"/>
+      <rgbColor rgb="FF80FF80"/>
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
@@ -561,7 +856,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Foglio1!$A$2:$A$4</c:f>
+              <c:f>Risultati!$A$2:$A$4</c:f>
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
@@ -578,7 +873,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Foglio1!$B$2:$B$4</c:f>
+              <c:f>Risultati!$B$2:$B$4</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -597,12 +892,12 @@
         </c:ser>
         <c:gapWidth val="100"/>
         <c:shape val="box"/>
-        <c:axId val="57980357"/>
-        <c:axId val="27227936"/>
+        <c:axId val="50837818"/>
+        <c:axId val="54883118"/>
         <c:axId val="0"/>
       </c:bar3DChart>
       <c:catAx>
-        <c:axId val="57980357"/>
+        <c:axId val="50837818"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -635,7 +930,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="27227936"/>
+        <c:crossAx val="54883118"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -643,7 +938,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="27227936"/>
+        <c:axId val="54883118"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="100"/>
@@ -686,7 +981,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="57980357"/>
+        <c:crossAx val="50837818"/>
         <c:crossesAt val="1"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1231,7 +1526,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Foglio1!$A$5:$A$14</c:f>
+              <c:f>Risultati!$A$5:$A$14</c:f>
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
@@ -1269,7 +1564,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Foglio1!$B$5:$B$14</c:f>
+              <c:f>Risultati!$B$5:$B$14</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -1309,12 +1604,12 @@
         </c:ser>
         <c:gapWidth val="100"/>
         <c:shape val="box"/>
-        <c:axId val="39084625"/>
-        <c:axId val="58546082"/>
+        <c:axId val="39164547"/>
+        <c:axId val="50354801"/>
         <c:axId val="0"/>
       </c:bar3DChart>
       <c:catAx>
-        <c:axId val="39084625"/>
+        <c:axId val="39164547"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1347,7 +1642,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="58546082"/>
+        <c:crossAx val="50354801"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1355,7 +1650,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="58546082"/>
+        <c:axId val="50354801"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="100"/>
@@ -1398,7 +1693,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="39084625"/>
+        <c:crossAx val="39164547"/>
         <c:crossesAt val="1"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1525,7 +1820,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Foglio1!$A$15:$A$19</c:f>
+              <c:f>Risultati!$A$15:$A$19</c:f>
               <c:strCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
@@ -1548,7 +1843,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Foglio1!$B$15:$B$19</c:f>
+              <c:f>Risultati!$B$15:$B$19</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
@@ -1571,11 +1866,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="63606581"/>
-        <c:axId val="60085722"/>
+        <c:axId val="49828442"/>
+        <c:axId val="39647775"/>
       </c:radarChart>
       <c:catAx>
-        <c:axId val="63606581"/>
+        <c:axId val="49828442"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1606,7 +1901,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="60085722"/>
+        <c:crossAx val="39647775"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1614,7 +1909,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="60085722"/>
+        <c:axId val="39647775"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="100"/>
@@ -1657,7 +1952,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="63606581"/>
+        <c:crossAx val="49828442"/>
         <c:crossesAt val="1"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1885,7 +2180,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Foglio1!$A$20:$A$22</c:f>
+              <c:f>Risultati!$A$20:$A$22</c:f>
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
@@ -1902,7 +2197,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Foglio1!$B$20:$B$22</c:f>
+              <c:f>Risultati!$B$20:$B$22</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -2054,10 +2349,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.1875"/>
-          <c:y val="0.191666666666667"/>
-          <c:w val="0.62490625"/>
-          <c:h val="0.666166666666667"/>
+          <c:x val="0.187511719482468"/>
+          <c:y val="0.191730576858953"/>
+          <c:w val="0.624882805175324"/>
+          <c:h val="0.666055351783928"/>
         </c:manualLayout>
       </c:layout>
       <c:bar3DChart>
@@ -2069,7 +2364,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Foglio1!$A$1</c:f>
+              <c:f>Risultati!$A$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2169,7 +2464,7 @@
           </c:dLbls>
           <c:val>
             <c:numRef>
-              <c:f>Foglio1!$B$1</c:f>
+              <c:f>Risultati!$B$1</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
@@ -2182,12 +2477,12 @@
         </c:ser>
         <c:gapWidth val="100"/>
         <c:shape val="box"/>
-        <c:axId val="61365308"/>
-        <c:axId val="66388280"/>
+        <c:axId val="38246914"/>
+        <c:axId val="98674786"/>
         <c:axId val="0"/>
       </c:bar3DChart>
       <c:catAx>
-        <c:axId val="61365308"/>
+        <c:axId val="38246914"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2220,7 +2515,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="66388280"/>
+        <c:crossAx val="98674786"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2228,7 +2523,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="66388280"/>
+        <c:axId val="98674786"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="100"/>
@@ -2271,7 +2566,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="61365308"/>
+        <c:crossAx val="38246914"/>
         <c:crossesAt val="0"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3391,9 +3686,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>79560</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>360</xdr:rowOff>
+      <xdr:colOff>78840</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>161640</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3402,7 +3697,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="0" y="0"/>
-        <a:ext cx="5758920" cy="3238920"/>
+        <a:ext cx="5758200" cy="3238200"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3421,9 +3716,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>148320</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>360</xdr:rowOff>
+      <xdr:colOff>147600</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>161640</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3432,7 +3727,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="5758560" y="0"/>
-        <a:ext cx="5758920" cy="3238920"/>
+        <a:ext cx="5758200" cy="3238200"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3451,9 +3746,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>79560</xdr:colOff>
+      <xdr:colOff>78840</xdr:colOff>
       <xdr:row>40</xdr:row>
-      <xdr:rowOff>1800</xdr:rowOff>
+      <xdr:rowOff>1080</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3462,7 +3757,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="0" y="3240000"/>
-        <a:ext cx="5758920" cy="3238920"/>
+        <a:ext cx="5758200" cy="3238200"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3481,9 +3776,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>148320</xdr:colOff>
+      <xdr:colOff>147600</xdr:colOff>
       <xdr:row>40</xdr:row>
-      <xdr:rowOff>1800</xdr:rowOff>
+      <xdr:rowOff>1080</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3492,7 +3787,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="5758560" y="3240000"/>
-        <a:ext cx="5758920" cy="3238920"/>
+        <a:ext cx="5758200" cy="3238200"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3511,9 +3806,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>150480</xdr:colOff>
+      <xdr:colOff>149760</xdr:colOff>
       <xdr:row>53</xdr:row>
-      <xdr:rowOff>57600</xdr:rowOff>
+      <xdr:rowOff>56880</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3522,7 +3817,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="0" y="6480000"/>
-        <a:ext cx="11519640" cy="2159640"/>
+        <a:ext cx="11518920" cy="2158920"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -5128,9 +5423,736 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1"/>
+  <dimension ref="A1:F71"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="3" width="40.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="3" width="30.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="15.32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="3" width="25.54"/>
+  </cols>
+  <sheetData>
+    <row r="1" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" s="11"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="12"/>
+    </row>
+    <row r="3" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" s="11"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="11"/>
+      <c r="F3" s="12"/>
+    </row>
+    <row r="4" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4" s="11"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="11"/>
+      <c r="E4" s="11"/>
+      <c r="F4" s="12"/>
+    </row>
+    <row r="5" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" s="11"/>
+      <c r="C5" s="12"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="12"/>
+    </row>
+    <row r="6" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" s="11"/>
+      <c r="C6" s="12"/>
+      <c r="D6" s="11"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="12"/>
+    </row>
+    <row r="7" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" s="11"/>
+      <c r="C7" s="12"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="12"/>
+    </row>
+    <row r="8" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" s="11"/>
+      <c r="C8" s="12"/>
+      <c r="D8" s="11"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="12"/>
+    </row>
+    <row r="9" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="B9" s="11"/>
+      <c r="C9" s="12"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="12"/>
+    </row>
+    <row r="10" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" s="11"/>
+      <c r="C10" s="12"/>
+      <c r="D10" s="11"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="12"/>
+    </row>
+    <row r="11" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="B11" s="11"/>
+      <c r="C11" s="12"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="12"/>
+    </row>
+    <row r="12" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="B12" s="11"/>
+      <c r="C12" s="12"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="12"/>
+    </row>
+    <row r="13" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="B13" s="11"/>
+      <c r="C13" s="12"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="12"/>
+    </row>
+    <row r="14" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="B14" s="11"/>
+      <c r="C14" s="12"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="11"/>
+      <c r="F14" s="12"/>
+    </row>
+    <row r="15" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="B15" s="11"/>
+      <c r="C15" s="12"/>
+      <c r="D15" s="11"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="12"/>
+    </row>
+    <row r="16" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="B16" s="11"/>
+      <c r="C16" s="12"/>
+      <c r="D16" s="11"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="12"/>
+    </row>
+    <row r="17" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B17" s="11"/>
+      <c r="C17" s="12"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="12"/>
+    </row>
+    <row r="18" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="B18" s="11"/>
+      <c r="C18" s="12"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="12"/>
+    </row>
+    <row r="19" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="B19" s="11"/>
+      <c r="C19" s="12"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="12"/>
+    </row>
+    <row r="20" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="B20" s="11"/>
+      <c r="C20" s="12"/>
+      <c r="D20" s="11"/>
+      <c r="E20" s="11"/>
+      <c r="F20" s="12"/>
+    </row>
+    <row r="21" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="B21" s="11"/>
+      <c r="C21" s="12"/>
+      <c r="D21" s="11"/>
+      <c r="E21" s="11"/>
+      <c r="F21" s="12"/>
+    </row>
+    <row r="22" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="B22" s="11"/>
+      <c r="C22" s="12"/>
+      <c r="D22" s="11"/>
+      <c r="E22" s="11"/>
+      <c r="F22" s="12"/>
+    </row>
+    <row r="23" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="B23" s="11"/>
+      <c r="C23" s="12"/>
+      <c r="D23" s="11"/>
+      <c r="E23" s="11"/>
+      <c r="F23" s="12"/>
+    </row>
+    <row r="24" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="B24" s="11"/>
+      <c r="C24" s="12"/>
+      <c r="D24" s="11"/>
+      <c r="E24" s="11"/>
+      <c r="F24" s="12"/>
+    </row>
+    <row r="25" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="B25" s="11"/>
+      <c r="C25" s="12"/>
+      <c r="D25" s="11"/>
+      <c r="E25" s="11"/>
+      <c r="F25" s="12"/>
+    </row>
+    <row r="26" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="B26" s="11"/>
+      <c r="C26" s="12"/>
+      <c r="D26" s="11"/>
+      <c r="E26" s="11"/>
+      <c r="F26" s="12"/>
+    </row>
+    <row r="27" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="B27" s="11"/>
+      <c r="C27" s="12"/>
+      <c r="D27" s="11"/>
+      <c r="E27" s="11"/>
+      <c r="F27" s="12"/>
+    </row>
+    <row r="28" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="B28" s="11"/>
+      <c r="C28" s="12"/>
+      <c r="D28" s="11"/>
+      <c r="E28" s="11"/>
+      <c r="F28" s="12"/>
+    </row>
+    <row r="29" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="B29" s="11"/>
+      <c r="C29" s="12"/>
+      <c r="D29" s="11"/>
+      <c r="E29" s="11"/>
+      <c r="F29" s="12"/>
+    </row>
+    <row r="30" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="B30" s="11"/>
+      <c r="C30" s="12"/>
+      <c r="D30" s="11"/>
+      <c r="E30" s="11"/>
+      <c r="F30" s="12"/>
+    </row>
+    <row r="31" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="B31" s="11"/>
+      <c r="C31" s="12"/>
+      <c r="D31" s="11"/>
+      <c r="E31" s="11"/>
+      <c r="F31" s="12"/>
+    </row>
+    <row r="32" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="B32" s="11"/>
+      <c r="C32" s="12"/>
+      <c r="D32" s="11"/>
+      <c r="E32" s="11"/>
+      <c r="F32" s="12"/>
+    </row>
+    <row r="33" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="B33" s="11"/>
+      <c r="C33" s="12"/>
+      <c r="D33" s="11"/>
+      <c r="E33" s="11"/>
+      <c r="F33" s="12"/>
+    </row>
+    <row r="34" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="B34" s="11"/>
+      <c r="C34" s="12"/>
+      <c r="D34" s="11"/>
+      <c r="E34" s="11"/>
+      <c r="F34" s="12"/>
+    </row>
+    <row r="35" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="B35" s="11"/>
+      <c r="C35" s="12"/>
+      <c r="D35" s="11"/>
+      <c r="E35" s="11"/>
+      <c r="F35" s="12"/>
+    </row>
+    <row r="36" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="B36" s="11"/>
+      <c r="C36" s="12"/>
+      <c r="D36" s="11"/>
+      <c r="E36" s="11"/>
+      <c r="F36" s="12"/>
+    </row>
+    <row r="37" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="B37" s="11"/>
+      <c r="C37" s="12"/>
+      <c r="D37" s="11"/>
+      <c r="E37" s="11"/>
+      <c r="F37" s="12"/>
+    </row>
+    <row r="38" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="14" t="s">
+        <v>63</v>
+      </c>
+      <c r="B38" s="11"/>
+      <c r="C38" s="12"/>
+      <c r="D38" s="11"/>
+      <c r="E38" s="11"/>
+      <c r="F38" s="12"/>
+    </row>
+    <row r="39" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="B39" s="11"/>
+      <c r="C39" s="12"/>
+      <c r="D39" s="11"/>
+      <c r="E39" s="11"/>
+      <c r="F39" s="12"/>
+    </row>
+    <row r="40" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="B40" s="11"/>
+      <c r="C40" s="12"/>
+      <c r="D40" s="11"/>
+      <c r="E40" s="11"/>
+      <c r="F40" s="12"/>
+    </row>
+    <row r="41" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="B41" s="11"/>
+      <c r="C41" s="12"/>
+      <c r="D41" s="11"/>
+      <c r="E41" s="11"/>
+      <c r="F41" s="12"/>
+    </row>
+    <row r="42" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="B42" s="11"/>
+      <c r="C42" s="12"/>
+      <c r="D42" s="11"/>
+      <c r="E42" s="11"/>
+      <c r="F42" s="12"/>
+    </row>
+    <row r="43" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="B43" s="11"/>
+      <c r="C43" s="12"/>
+      <c r="D43" s="11"/>
+      <c r="E43" s="11"/>
+      <c r="F43" s="12"/>
+    </row>
+    <row r="44" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="B44" s="11"/>
+      <c r="C44" s="12"/>
+      <c r="D44" s="11"/>
+      <c r="E44" s="11"/>
+      <c r="F44" s="12"/>
+    </row>
+    <row r="45" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45" s="11"/>
+      <c r="C45" s="12"/>
+      <c r="D45" s="11"/>
+      <c r="E45" s="11"/>
+      <c r="F45" s="12"/>
+    </row>
+    <row r="46" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46" s="11"/>
+      <c r="C46" s="12"/>
+      <c r="D46" s="11"/>
+      <c r="E46" s="11"/>
+      <c r="F46" s="12"/>
+    </row>
+    <row r="47" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="B47" s="11"/>
+      <c r="C47" s="12"/>
+      <c r="D47" s="11"/>
+      <c r="E47" s="11"/>
+      <c r="F47" s="12"/>
+    </row>
+    <row r="48" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="16" t="s">
+        <v>73</v>
+      </c>
+      <c r="B48" s="11"/>
+      <c r="C48" s="12"/>
+      <c r="D48" s="11"/>
+      <c r="E48" s="11"/>
+      <c r="F48" s="12"/>
+    </row>
+    <row r="49" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="B49" s="11"/>
+      <c r="C49" s="12"/>
+      <c r="D49" s="11"/>
+      <c r="E49" s="11"/>
+      <c r="F49" s="12"/>
+    </row>
+    <row r="50" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="16" t="s">
+        <v>75</v>
+      </c>
+      <c r="B50" s="11"/>
+      <c r="C50" s="12"/>
+      <c r="D50" s="11"/>
+      <c r="E50" s="11"/>
+      <c r="F50" s="12"/>
+    </row>
+    <row r="51" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="14" t="s">
+        <v>76</v>
+      </c>
+      <c r="B51" s="11"/>
+      <c r="C51" s="12"/>
+      <c r="D51" s="11"/>
+      <c r="E51" s="11"/>
+      <c r="F51" s="12"/>
+    </row>
+    <row r="52" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="B52" s="11"/>
+      <c r="C52" s="12"/>
+      <c r="D52" s="11"/>
+      <c r="E52" s="11"/>
+      <c r="F52" s="12"/>
+    </row>
+    <row r="53" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="B53" s="11"/>
+      <c r="C53" s="12"/>
+      <c r="D53" s="11"/>
+      <c r="E53" s="11"/>
+      <c r="F53" s="12"/>
+    </row>
+    <row r="54" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="B54" s="11"/>
+      <c r="C54" s="12"/>
+      <c r="D54" s="11"/>
+      <c r="E54" s="11"/>
+      <c r="F54" s="12"/>
+    </row>
+    <row r="55" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="B55" s="11"/>
+      <c r="C55" s="12"/>
+      <c r="D55" s="11"/>
+      <c r="E55" s="11"/>
+      <c r="F55" s="12"/>
+    </row>
+    <row r="56" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="B56" s="11"/>
+      <c r="C56" s="12"/>
+      <c r="D56" s="11"/>
+      <c r="E56" s="11"/>
+      <c r="F56" s="12"/>
+    </row>
+    <row r="57" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="B57" s="11"/>
+      <c r="C57" s="12"/>
+      <c r="D57" s="11"/>
+      <c r="E57" s="11"/>
+      <c r="F57" s="12"/>
+    </row>
+    <row r="58" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="B58" s="11"/>
+      <c r="C58" s="12"/>
+      <c r="D58" s="11"/>
+      <c r="E58" s="11"/>
+      <c r="F58" s="12"/>
+    </row>
+    <row r="59" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="B59" s="11"/>
+      <c r="C59" s="12"/>
+      <c r="D59" s="11"/>
+      <c r="E59" s="11"/>
+      <c r="F59" s="12"/>
+    </row>
+    <row r="60" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="15" t="s">
+        <v>85</v>
+      </c>
+      <c r="B60" s="11"/>
+      <c r="C60" s="12"/>
+      <c r="D60" s="11"/>
+      <c r="E60" s="11"/>
+      <c r="F60" s="12"/>
+    </row>
+    <row r="61" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="B61" s="11"/>
+      <c r="C61" s="12"/>
+      <c r="D61" s="11"/>
+      <c r="E61" s="11"/>
+      <c r="F61" s="12"/>
+    </row>
+    <row r="62" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="B62" s="11"/>
+      <c r="C62" s="12"/>
+      <c r="D62" s="11"/>
+      <c r="E62" s="11"/>
+      <c r="F62" s="12"/>
+    </row>
+    <row r="63" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="B63" s="11"/>
+      <c r="C63" s="12"/>
+      <c r="D63" s="11"/>
+      <c r="E63" s="11"/>
+      <c r="F63" s="12"/>
+    </row>
+    <row r="64" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="B64" s="11"/>
+      <c r="C64" s="12"/>
+      <c r="D64" s="11"/>
+      <c r="E64" s="11"/>
+      <c r="F64" s="12"/>
+    </row>
+    <row r="65" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="B65" s="11"/>
+      <c r="C65" s="12"/>
+      <c r="D65" s="11"/>
+      <c r="E65" s="11"/>
+      <c r="F65" s="12"/>
+    </row>
+    <row r="66" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="B66" s="11"/>
+      <c r="C66" s="12"/>
+      <c r="D66" s="11"/>
+      <c r="E66" s="11"/>
+      <c r="F66" s="12"/>
+    </row>
+    <row r="67" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="B67" s="11"/>
+      <c r="C67" s="12"/>
+      <c r="D67" s="11"/>
+      <c r="E67" s="11"/>
+      <c r="F67" s="12"/>
+    </row>
+    <row r="68" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="14" t="s">
+        <v>93</v>
+      </c>
+      <c r="B68" s="11"/>
+      <c r="C68" s="12"/>
+      <c r="D68" s="11"/>
+      <c r="E68" s="11"/>
+      <c r="F68" s="12"/>
+    </row>
+    <row r="69" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A69" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="B69" s="11"/>
+      <c r="C69" s="12"/>
+      <c r="D69" s="11"/>
+      <c r="E69" s="11"/>
+      <c r="F69" s="12"/>
+    </row>
+    <row r="70" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A70" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="B70" s="11"/>
+      <c r="C70" s="12"/>
+      <c r="D70" s="11"/>
+      <c r="E70" s="11"/>
+      <c r="F70" s="12"/>
+    </row>
+    <row r="71" s="13" customFormat="true" ht="85.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A71" s="15" t="s">
+        <v>96</v>
+      </c>
+      <c r="B71" s="11"/>
+      <c r="C71" s="12"/>
+      <c r="D71" s="11"/>
+      <c r="E71" s="11"/>
+      <c r="F71" s="12"/>
+    </row>
+  </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>